<commit_message>
Add BBVA crédito and MSI row from VANS - 1 workbook
Second BBVA row from MONETIZAR_-_VANS_-_1 (Escenario 1): debit, credit,
AMEX, international commissions and MSI surcharges 3x-18x.

Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -71,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,6 +90,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -632,6 +641,67 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>VANS - 1</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>77945500</v>
+      </c>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="9" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0.0142</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0.0202</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>0.0202</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>0.0493</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>0.0842</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>0.1174</v>
+      </c>
+      <c r="P3" s="9" t="n">
+        <v>0.1491</v>
+      </c>
+      <c r="Q3" s="9" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="R3" s="9" t="n"/>
+      <c r="S3" s="6" t="inlineStr">
+        <is>
+          <t>Origen: MONETIZAR_-_VANS_-_1.xlsx, hoja 'Escenario 1'. TPV = B2 ('Grupo'). Débito = B20 (TD), Crédito = B21 (TC), AMEX = B22, Internacional = B23. Sobretasas MSI = L21:L25 (3x a 18x). Base de tasa TC = B21 (2.02%). 24x no aparece. Ticket promedio vacío. Nota: los valores de BBVA no coinciden con el archivo anterior (TD 1.5% vs 1.42%, MSI más altos).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark VANS - 1 BBVA rates as current
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -587,64 +587,64 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>VANS</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>VANS (NO VIGENTE)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="8" t="n">
         <v>77945500</v>
       </c>
       <c r="D2" s="4" t="n"/>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="9" t="n">
         <v>0.43</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="9" t="n">
         <v>0.51</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="9" t="n">
         <v>0.02</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
-      <c r="M2" s="5" t="n">
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n"/>
+      <c r="L2" s="9" t="n"/>
+      <c r="M2" s="9" t="n">
         <v>0.035</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="9" t="n">
         <v>0.04</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="9" t="n">
         <v>0.065</v>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="9" t="n">
         <v>0.095</v>
       </c>
-      <c r="Q2" s="5" t="n">
+      <c r="Q2" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="R2" s="5" t="n"/>
+      <c r="R2" s="9" t="n"/>
       <c r="S2" s="6" t="inlineStr">
         <is>
-          <t>Origen: hoja 'Monetización'. TPV = B3 (etiquetado 'Grupo', confirmar). Ticket promedio vacío (B5). Débito = B25. MSI = sobretasas L36:L40 (3x usa fila 36; 3x Citi en L35 también 3.5%). Crédito/AMEX/Internacional sin tasa en el archivo (base TC en B36 vacía). 24x no aparece en el archivo. MSI share (B13) = 4%, no mapeado a columna.</t>
+          <t>NO VIGENTE (reemplazada por VANS - 1). Origen: hoja 'Monetización'. TPV = B3 (etiquetado 'Grupo', confirmar). Ticket promedio vacío (B5). Débito = B25. MSI = sobretasas L36:L40 (3x usa fila 36; 3x Citi en L35 también 3.5%). Crédito/AMEX/Internacional sin tasa en el archivo (base TC en B36 vacía). 24x no aparece en el archivo. MSI share (B13) = 4%, no mapeado a columna.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>VANS - 1</t>
+          <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -698,7 +698,7 @@
       <c r="R3" s="9" t="n"/>
       <c r="S3" s="6" t="inlineStr">
         <is>
-          <t>Origen: MONETIZAR_-_VANS_-_1.xlsx, hoja 'Escenario 1'. TPV = B2 ('Grupo'). Débito = B20 (TD), Crédito = B21 (TC), AMEX = B22, Internacional = B23. Sobretasas MSI = L21:L25 (3x a 18x). Base de tasa TC = B21 (2.02%). 24x no aparece. Ticket promedio vacío. Nota: los valores de BBVA no coinciden con el archivo anterior (TD 1.5% vs 1.42%, MSI más altos).</t>
+          <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1.xlsx, hoja 'Escenario 1'. TPV = B2 ('Grupo'). Débito = B20 (TD), Crédito = B21 (TC), AMEX = B22, Internacional = B23. Sobretasas MSI = L21:L25 (3x a 18x). Base de tasa TC = B21 (2.02%). 24x no aparece. Ticket promedio vacío. Nota: los valores de BBVA no coinciden con el archivo anterior (TD 1.5% vs 1.42%, MSI más altos).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add San Angel INN, VEANNA and Aguillon competitor rows; Industria column
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -42,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,12 +76,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -90,15 +98,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -465,28 +464,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="9" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="70" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="80" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -502,203 +502,490 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Industria (llenar manual)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>TPV</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ticket promedio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Share TD</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Share TC</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Share AMEX</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Share Internacional</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Comisión Débito</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Comisión Crédito</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Comisión AMEX</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Comisión Internacional</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>3x</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>6x</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>9x</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>12x</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>18x</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>24x</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Notas / celdas origen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="4" t="n">
         <v>77945500</v>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="6" t="n">
         <v>0.43</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="G2" s="6" t="n">
         <v>0.51</v>
       </c>
-      <c r="G2" s="9" t="n">
+      <c r="H2" s="6" t="n">
         <v>0.02</v>
       </c>
-      <c r="H2" s="9" t="n">
+      <c r="I2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="9" t="n">
+      <c r="J2" s="6" t="n">
         <v>0.015</v>
       </c>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="n">
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n">
         <v>0.035</v>
       </c>
-      <c r="N2" s="9" t="n">
+      <c r="O2" s="6" t="n">
         <v>0.04</v>
       </c>
-      <c r="O2" s="9" t="n">
+      <c r="P2" s="6" t="n">
         <v>0.065</v>
       </c>
-      <c r="P2" s="9" t="n">
+      <c r="Q2" s="6" t="n">
         <v>0.095</v>
       </c>
-      <c r="Q2" s="9" t="n">
+      <c r="R2" s="6" t="n">
         <v>0.15</v>
       </c>
-      <c r="R2" s="9" t="n"/>
-      <c r="S2" s="6" t="inlineStr">
-        <is>
-          <t>NO VIGENTE (reemplazada por VANS - 1). Origen: hoja 'Monetización'. TPV = B3 (etiquetado 'Grupo', confirmar). Ticket promedio vacío (B5). Débito = B25. MSI = sobretasas L36:L40 (3x usa fila 36; 3x Citi en L35 también 3.5%). Crédito/AMEX/Internacional sin tasa en el archivo (base TC en B36 vacía). 24x no aparece en el archivo. MSI share (B13) = 4%, no mapeado a columna.</t>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="7" t="inlineStr">
+        <is>
+          <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="4" t="n">
         <v>77945500</v>
       </c>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="6" t="n">
         <v>0.43</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="G3" s="6" t="n">
         <v>0.51</v>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="H3" s="6" t="n">
         <v>0.02</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="I3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="J3" s="6" t="n">
         <v>0.0142</v>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="K3" s="6" t="n">
         <v>0.0202</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="L3" s="6" t="n">
         <v>0.03</v>
       </c>
-      <c r="L3" s="9" t="n">
+      <c r="M3" s="6" t="n">
         <v>0.0202</v>
       </c>
-      <c r="M3" s="9" t="n">
+      <c r="N3" s="6" t="n">
         <v>0.0493</v>
       </c>
-      <c r="N3" s="9" t="n">
+      <c r="O3" s="6" t="n">
         <v>0.0842</v>
       </c>
-      <c r="O3" s="9" t="n">
+      <c r="P3" s="6" t="n">
         <v>0.1174</v>
       </c>
-      <c r="P3" s="9" t="n">
+      <c r="Q3" s="6" t="n">
         <v>0.1491</v>
       </c>
-      <c r="Q3" s="9" t="n">
+      <c r="R3" s="6" t="n">
         <v>0.19</v>
       </c>
-      <c r="R3" s="9" t="n"/>
-      <c r="S3" s="6" t="inlineStr">
-        <is>
-          <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1.xlsx, hoja 'Escenario 1'. TPV = B2 ('Grupo'). Débito = B20 (TD), Crédito = B21 (TC), AMEX = B22, Internacional = B23. Sobretasas MSI = L21:L25 (3x a 18x). Base de tasa TC = B21 (2.02%). 24x no aparece. Ticket promedio vacío. Nota: los valores de BBVA no coinciden con el archivo anterior (TD 1.5% vs 1.42%, MSI más altos).</t>
+      <c r="S3" s="6" t="n"/>
+      <c r="T3" s="7" t="inlineStr">
+        <is>
+          <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>San Angel INN 2 terminales</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="4" t="n">
+        <v>9213568.4673</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>555</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0.2758</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.1315</v>
+      </c>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="N4" s="6" t="n">
+        <v>0.0501</v>
+      </c>
+      <c r="O4" s="6" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="P4" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Q4" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S4" s="6" t="n"/>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>San Angel INN 2 terminales</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MIFEL</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="4" t="n">
+        <v>11838651.3927</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>555</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0.3652</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="n"/>
+      <c r="N5" s="6" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S5" s="6" t="n"/>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VEANNA</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="4" t="n">
+        <v>36864986.512</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>544</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0.6686303192319475</v>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n">
+        <v>0.01490860168417793</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M6" s="6" t="n"/>
+      <c r="N6" s="6" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="6" t="n"/>
+      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="6" t="n"/>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VEANNA</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="4" t="n">
+        <v>1940262.448</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>544</v>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n">
+        <v>0.0136</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.0181</v>
+      </c>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="6" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>0.0735</v>
+      </c>
+      <c r="P7" s="6" t="n"/>
+      <c r="Q7" s="6" t="n"/>
+      <c r="R7" s="6" t="n"/>
+      <c r="S7" s="6" t="n"/>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Aguillon</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CLIP</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="4" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>0.0457</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>0.0757</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>0.1107</v>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>0.1277</v>
+      </c>
+      <c r="R8" s="6" t="n"/>
+      <c r="S8" s="6" t="n"/>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, confirmar. Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Auna, HangTen 2 and Caso 3 competitor rows
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -989,6 +1004,316 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Auna</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="10" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="12" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O9" s="12" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="P9" s="12" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="Q9" s="12" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="R9" s="12" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="S9" s="12" t="n"/>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (encabezado 'Anual', confirmar base). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Auna</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Fiserv</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="10" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="12" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="L10" s="12" t="n"/>
+      <c r="M10" s="12" t="n"/>
+      <c r="N10" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P10" s="12" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R10" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S10" s="12" t="n"/>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>HangTen 2</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="10" t="n">
+        <v>136100110.57</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>555</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>0.6713</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>0.3075</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.0145</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O11" s="12" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="P11" s="12" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q11" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R11" s="12" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="S11" s="12" t="n"/>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Origen: 'Monetizacion 0.45%' (encabezado 'ANUAL'). TPV = B3 (anual). Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>HangTen 2</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Fiserv</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="10" t="n">
+        <v>94010839.39</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>555</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>0.6605</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>0.3389</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.0144</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>0.0179</v>
+      </c>
+      <c r="L12" s="12" t="n"/>
+      <c r="M12" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O12" s="12" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="P12" s="12" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R12" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S12" s="12" t="n"/>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV = B4. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Caso 3 soluciones</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Fiserv</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="10" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>555</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O13" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P13" s="12" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q13" s="12" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R13" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S13" s="12" t="n"/>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Lineas (BBVA, Fiserv) and Vertex (BBVA, Banamex) competitor rows
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -479,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -607,55 +622,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="4" t="n">
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="10" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="6" t="n">
+      <c r="E2" s="11" t="n"/>
+      <c r="F2" s="12" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="12" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="12" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="6" t="n">
+      <c r="J2" s="12" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="6" t="n"/>
-      <c r="L2" s="6" t="n"/>
-      <c r="M2" s="6" t="n"/>
-      <c r="N2" s="6" t="n">
+      <c r="K2" s="12" t="n"/>
+      <c r="L2" s="12" t="n"/>
+      <c r="M2" s="12" t="n"/>
+      <c r="N2" s="12" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="O2" s="12" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="6" t="n">
+      <c r="P2" s="12" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="6" t="n">
+      <c r="Q2" s="12" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="6" t="n">
+      <c r="R2" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="6" t="n"/>
+      <c r="S2" s="12" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -663,61 +678,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="4" t="n">
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="10" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="n">
+      <c r="E3" s="11" t="n"/>
+      <c r="F3" s="12" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="12" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="12" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="12" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="K3" s="12" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="L3" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="M3" s="12" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="N3" s="12" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="O3" s="12" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="6" t="n">
+      <c r="P3" s="12" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="6" t="n">
+      <c r="Q3" s="12" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="6" t="n">
+      <c r="R3" s="12" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="6" t="n"/>
+      <c r="S3" s="12" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -725,61 +740,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="4" t="n">
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="10" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="11" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="12" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="12" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n">
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="12" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="K4" s="12" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="L4" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="M4" s="12" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="N4" s="12" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="O4" s="12" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="6" t="n">
+      <c r="P4" s="12" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="6" t="n">
+      <c r="Q4" s="12" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="6" t="n">
+      <c r="R4" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="6" t="n"/>
+      <c r="S4" s="12" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -787,59 +802,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="4" t="n">
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="10" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="11" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="12" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="12" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="12" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="12" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="K5" s="12" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="6" t="n"/>
-      <c r="M5" s="6" t="n"/>
-      <c r="N5" s="6" t="n">
+      <c r="L5" s="12" t="n"/>
+      <c r="M5" s="12" t="n"/>
+      <c r="N5" s="12" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="O5" s="12" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="P5" s="12" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="Q5" s="12" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="R5" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="6" t="n"/>
+      <c r="S5" s="12" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -847,53 +862,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="4" t="n">
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="10" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="11" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="12" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="6" t="n">
+      <c r="J6" s="12" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="6" t="n">
+      <c r="K6" s="12" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="6" t="n">
+      <c r="L6" s="12" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="6" t="n"/>
-      <c r="N6" s="6" t="n">
+      <c r="M6" s="12" t="n"/>
+      <c r="N6" s="12" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="O6" s="12" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="6" t="n"/>
-      <c r="S6" s="6" t="n"/>
+      <c r="P6" s="12" t="n"/>
+      <c r="Q6" s="12" t="n"/>
+      <c r="R6" s="12" t="n"/>
+      <c r="S6" s="12" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -901,45 +916,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="4" t="n">
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="10" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="11" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n">
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="12" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="12" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="6" t="n">
+      <c r="K7" s="12" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="6" t="n"/>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="n">
+      <c r="L7" s="12" t="n"/>
+      <c r="M7" s="12" t="n"/>
+      <c r="N7" s="12" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="O7" s="12" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="6" t="n"/>
-      <c r="R7" s="6" t="n"/>
-      <c r="S7" s="6" t="n"/>
+      <c r="P7" s="12" t="n"/>
+      <c r="Q7" s="12" t="n"/>
+      <c r="R7" s="12" t="n"/>
+      <c r="S7" s="12" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -947,57 +962,57 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="4" t="n">
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="11" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="12" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n">
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="6" t="n">
+      <c r="K8" s="12" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="6" t="n">
+      <c r="L8" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="6" t="n">
+      <c r="M8" s="12" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="6" t="n">
+      <c r="N8" s="12" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="6" t="n">
+      <c r="O8" s="12" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="6" t="n">
+      <c r="P8" s="12" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="6" t="n">
+      <c r="Q8" s="12" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="6" t="n"/>
-      <c r="S8" s="6" t="n"/>
+      <c r="R8" s="12" t="n"/>
+      <c r="S8" s="12" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, confirmar. Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos.</t>
@@ -1314,6 +1329,254 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Lineas</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="15" t="n">
+        <v>24619599.25</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>555</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J14" s="17" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="K14" s="17" t="n">
+        <v>0.0161</v>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="M14" s="17" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="N14" s="17" t="n">
+        <v>0.0501</v>
+      </c>
+      <c r="O14" s="17" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="P14" s="17" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Q14" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="R14" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S14" s="17" t="n"/>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo'. Merchant = CITI. TPV = B3 = B2/12 x C2 (B2 anual 295,435,191 / 12 x 100%). Shares TD B7, TC B8, Int B14. Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. 24x no aparece. Otras hojas: 'EscenarioPsycho' tiene TPV 32M y AMEX/Int distintos (2.6%/2.4%) y 3x 1.91%; 'Flujo Comp (2)' y '1.77-1.99' tienen tasas distintas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Lineas</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Fiserv</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="15" t="n">
+        <v>24619599.25</v>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>555</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J15" s="17" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="K15" s="17" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="17" t="n"/>
+      <c r="N15" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O15" s="17" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P15" s="17" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q15" s="17" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R15" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S15" s="17" t="n"/>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo', sección Fiserv. Mismo TPV y shares que BBVA. Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin AMEX/Internacional. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="15" t="n">
+        <v>5200000</v>
+      </c>
+      <c r="E16" s="16" t="n">
+        <v>555</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="17" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="L16" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M16" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="N16" s="17" t="n">
+        <v>0.0553</v>
+      </c>
+      <c r="O16" s="17" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="P16" s="17" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="Q16" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="R16" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S16" s="17" t="n"/>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion ' (con espacio). TPV = B2 (8M) x C3 (65%). Share TD B7, TC B8 (BBVA MSI 10%, B9, sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI K26:K30. 24x no aparece. Sin periodo en el archivo (confirmar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Banamex</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="15" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>555</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K17" s="17" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="L17" s="17" t="n"/>
+      <c r="M17" s="17" t="n"/>
+      <c r="N17" s="17" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O17" s="17" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P17" s="17" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q17" s="17" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R17" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S17" s="17" t="n"/>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion ', sección Banamex. TPV = B2 (8M) x C4 (35%). Share DEB Banamex B10 (TD), CRE B11 (TC). Débito B38, Crédito B39. Sobretasas MSI K39:K43. Sin AMEX/Internacional. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Florence, grupo_milano, Carlos Toys, Kaloni and Bobois competitor rows
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -494,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -622,55 +637,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="10" t="n">
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="15" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="11" t="n"/>
-      <c r="F2" s="12" t="n">
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="17" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="12" t="n">
+      <c r="G2" s="17" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="I2" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="12" t="n">
+      <c r="J2" s="17" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="12" t="n"/>
-      <c r="L2" s="12" t="n"/>
-      <c r="M2" s="12" t="n"/>
-      <c r="N2" s="12" t="n">
+      <c r="K2" s="17" t="n"/>
+      <c r="L2" s="17" t="n"/>
+      <c r="M2" s="17" t="n"/>
+      <c r="N2" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="12" t="n">
+      <c r="O2" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="12" t="n">
+      <c r="P2" s="17" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="12" t="n">
+      <c r="Q2" s="17" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="12" t="n">
+      <c r="R2" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="12" t="n"/>
+      <c r="S2" s="17" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -678,61 +693,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="10" t="n">
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="15" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="12" t="n">
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="17" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="G3" s="17" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="17" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="K3" s="17" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="L3" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="M3" s="17" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="12" t="n">
+      <c r="N3" s="17" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="12" t="n">
+      <c r="O3" s="17" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="12" t="n">
+      <c r="P3" s="17" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="12" t="n">
+      <c r="Q3" s="17" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="12" t="n">
+      <c r="R3" s="17" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="12" t="n"/>
+      <c r="S3" s="17" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -740,61 +755,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="10" t="n">
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="15" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="16" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="17" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="17" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n">
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="17" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="17" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="L4" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="M4" s="17" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="N4" s="17" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="12" t="n">
+      <c r="O4" s="17" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="12" t="n">
+      <c r="P4" s="17" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="12" t="n">
+      <c r="Q4" s="17" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="12" t="n">
+      <c r="R4" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="12" t="n"/>
+      <c r="S4" s="17" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -802,59 +817,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="10" t="n">
+      <c r="C5" s="14" t="n"/>
+      <c r="D5" s="15" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="16" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="17" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="17" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="17" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="17" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="17" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="12" t="n">
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="12" t="n">
+      <c r="O5" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="12" t="n">
+      <c r="P5" s="17" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="12" t="n">
+      <c r="Q5" s="17" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="12" t="n">
+      <c r="R5" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="12" t="n"/>
+      <c r="S5" s="17" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -862,53 +877,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="10" t="n">
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="15" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="16" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="17" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="12" t="n">
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="17" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="17" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="12" t="n">
+      <c r="M6" s="17" t="n"/>
+      <c r="N6" s="17" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="12" t="n">
+      <c r="O6" s="17" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="12" t="n"/>
-      <c r="Q6" s="12" t="n"/>
-      <c r="R6" s="12" t="n"/>
-      <c r="S6" s="12" t="n"/>
+      <c r="P6" s="17" t="n"/>
+      <c r="Q6" s="17" t="n"/>
+      <c r="R6" s="17" t="n"/>
+      <c r="S6" s="17" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -916,45 +931,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="10" t="n">
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="15" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="16" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="12" t="n"/>
-      <c r="I7" s="12" t="n"/>
-      <c r="J7" s="12" t="n">
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="17" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="12" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="12" t="n">
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
+      <c r="N7" s="17" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="12" t="n">
+      <c r="O7" s="17" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="12" t="n"/>
-      <c r="Q7" s="12" t="n"/>
-      <c r="R7" s="12" t="n"/>
-      <c r="S7" s="12" t="n"/>
+      <c r="P7" s="17" t="n"/>
+      <c r="Q7" s="17" t="n"/>
+      <c r="R7" s="17" t="n"/>
+      <c r="S7" s="17" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -962,57 +977,57 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="10" t="n">
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="15" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="16" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="17" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="17" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="n"/>
-      <c r="J8" s="12" t="n">
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="17" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="12" t="n">
+      <c r="L8" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="12" t="n">
+      <c r="M8" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="17" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="12" t="n">
+      <c r="O8" s="17" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="P8" s="17" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="12" t="n">
+      <c r="Q8" s="17" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="12" t="n"/>
-      <c r="S8" s="12" t="n"/>
+      <c r="R8" s="17" t="n"/>
+      <c r="S8" s="17" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, confirmar. Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos.</t>
@@ -1020,61 +1035,61 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="10" t="n">
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="15" t="n">
         <v>40000000</v>
       </c>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="12" t="n">
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="17" t="n">
         <v>0.29</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="17" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="17" t="n">
         <v>0.08</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="17" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="17" t="n">
         <v>0.0115</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="17" t="n">
         <v>0.0167</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="M9" s="17" t="n">
         <v>0.025</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="17" t="n">
         <v>0.032</v>
       </c>
-      <c r="O9" s="12" t="n">
+      <c r="O9" s="17" t="n">
         <v>0.048</v>
       </c>
-      <c r="P9" s="12" t="n">
+      <c r="P9" s="17" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q9" s="12" t="n">
+      <c r="Q9" s="17" t="n">
         <v>0.105</v>
       </c>
-      <c r="R9" s="12" t="n">
+      <c r="R9" s="17" t="n">
         <v>0.16</v>
       </c>
-      <c r="S9" s="12" t="n"/>
+      <c r="S9" s="17" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (encabezado 'Anual', confirmar base). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
@@ -1082,57 +1097,57 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="10" t="n">
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="15" t="n">
         <v>40000000</v>
       </c>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="12" t="n">
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="17" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H10" s="17" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="17" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="17" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="K10" s="17" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L10" s="12" t="n"/>
-      <c r="M10" s="12" t="n"/>
-      <c r="N10" s="12" t="n">
+      <c r="L10" s="17" t="n"/>
+      <c r="M10" s="17" t="n"/>
+      <c r="N10" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O10" s="12" t="n">
+      <c r="O10" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="P10" s="12" t="n">
+      <c r="P10" s="17" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q10" s="12" t="n">
+      <c r="Q10" s="17" t="n">
         <v>0.095</v>
       </c>
-      <c r="R10" s="12" t="n">
+      <c r="R10" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S10" s="12" t="n"/>
+      <c r="S10" s="17" t="n"/>
       <c r="T10" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece.</t>
@@ -1140,63 +1155,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="10" t="n">
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="15" t="n">
         <v>136100110.57</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="16" t="n">
         <v>555</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="17" t="n">
         <v>0.6713</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="17" t="n">
         <v>0.3075</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="17" t="n">
         <v>0.0212</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="17" t="n">
         <v>0.0145</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="K11" s="17" t="n">
         <v>0.018</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="L11" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="M11" s="17" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N11" s="12" t="n">
+      <c r="N11" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O11" s="12" t="n">
+      <c r="O11" s="17" t="n">
         <v>0.075</v>
       </c>
-      <c r="P11" s="12" t="n">
+      <c r="P11" s="17" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q11" s="12" t="n">
+      <c r="Q11" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="R11" s="12" t="n">
+      <c r="R11" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="S11" s="12" t="n"/>
+      <c r="S11" s="17" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%' (encabezado 'ANUAL'). TPV = B3 (anual). Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
@@ -1204,61 +1219,61 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="10" t="n">
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="15" t="n">
         <v>94010839.39</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="16" t="n">
         <v>555</v>
       </c>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="17" t="n">
         <v>0.6605</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="17" t="n">
         <v>0.3389</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="17" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="17" t="n">
         <v>0.0144</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="K12" s="17" t="n">
         <v>0.0179</v>
       </c>
-      <c r="L12" s="12" t="n"/>
-      <c r="M12" s="12" t="n">
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O12" s="12" t="n">
+      <c r="O12" s="17" t="n">
         <v>0.045</v>
       </c>
-      <c r="P12" s="12" t="n">
+      <c r="P12" s="17" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q12" s="12" t="n">
+      <c r="Q12" s="17" t="n">
         <v>0.095</v>
       </c>
-      <c r="R12" s="12" t="n">
+      <c r="R12" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S12" s="12" t="n"/>
+      <c r="S12" s="17" t="n"/>
       <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV = B4. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
@@ -1266,63 +1281,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Caso 3 soluciones</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="10" t="n">
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="15" t="n">
         <v>10000000</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="16" t="n">
         <v>555</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="17" t="n">
         <v>0.28</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="17" t="n">
         <v>0.01</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="I13" s="17" t="n">
         <v>0.01</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="J13" s="17" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="K13" s="17" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L13" s="12" t="n">
+      <c r="L13" s="17" t="n">
         <v>0.03</v>
       </c>
-      <c r="M13" s="12" t="n">
+      <c r="M13" s="17" t="n">
         <v>0.034</v>
       </c>
-      <c r="N13" s="12" t="n">
+      <c r="N13" s="17" t="n">
         <v>0.035</v>
       </c>
-      <c r="O13" s="12" t="n">
+      <c r="O13" s="17" t="n">
         <v>0.04</v>
       </c>
-      <c r="P13" s="12" t="n">
+      <c r="P13" s="17" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="12" t="n">
+      <c r="Q13" s="17" t="n">
         <v>0.095</v>
       </c>
-      <c r="R13" s="12" t="n">
+      <c r="R13" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="S13" s="12" t="n"/>
+      <c r="S13" s="17" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
@@ -1577,6 +1592,302 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Florence</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="20" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G18" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I18" s="22" t="n"/>
+      <c r="J18" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K18" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L18" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="22" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P18" s="22" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q18" s="22" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R18" s="22" t="n"/>
+      <c r="S18" s="22" t="n"/>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>grupo_milano</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="20" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H19" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I19" s="22" t="n"/>
+      <c r="J19" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K19" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L19" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="22" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O19" s="22" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P19" s="22" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q19" s="22" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R19" s="22" t="n"/>
+      <c r="S19" s="22" t="n"/>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Carlos Toys</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="20" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F20" s="22" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G20" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H20" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I20" s="22" t="n"/>
+      <c r="J20" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K20" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L20" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="22" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O20" s="22" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P20" s="22" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q20" s="22" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R20" s="22" t="n"/>
+      <c r="S20" s="22" t="n"/>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Kaloni</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="20" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H21" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I21" s="22" t="n"/>
+      <c r="J21" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="K21" s="22" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L21" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="22" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O21" s="22" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P21" s="22" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q21" s="22" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R21" s="22" t="n"/>
+      <c r="S21" s="22" t="n"/>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Bobois</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="20" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <v>800</v>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G22" s="22" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H22" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I22" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J22" s="22" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="K22" s="22" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="L22" s="22" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M22" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N22" s="22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O22" s="22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P22" s="22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q22" s="22" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="R22" s="22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S22" s="22" t="n"/>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Escenario 24 horas '. Competidor no nombrado ('Solución actual'). TPV = B2 (6M), ticket = B3. Shares TD B5, TC B6, AMEX B7, Internacional = Débito B8 + Crédito B9 (0.5% + 0.5%). MSI 0% (B10). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%) - ambos 3.0%. Sobretasas MSI K17:K22 (3x con Citi 5% y 3x 5%; 18x 18.9%). 24x no aparece. Otras hojas (Escenario 1, 48 horas, citi 3x, Hoja2) tienen valores distintos.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark Auna, HangTen 2 and CLIP TPV as monthly
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -637,55 +637,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="15" t="n">
+      <c r="C2" s="19" t="n"/>
+      <c r="D2" s="20" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="17" t="n">
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="22" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="17" t="n">
+      <c r="G2" s="22" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="17" t="n">
+      <c r="H2" s="22" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="17" t="n">
+      <c r="I2" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="17" t="n">
+      <c r="J2" s="22" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="17" t="n"/>
-      <c r="L2" s="17" t="n"/>
-      <c r="M2" s="17" t="n"/>
-      <c r="N2" s="17" t="n">
+      <c r="K2" s="22" t="n"/>
+      <c r="L2" s="22" t="n"/>
+      <c r="M2" s="22" t="n"/>
+      <c r="N2" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="17" t="n">
+      <c r="O2" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="17" t="n">
+      <c r="P2" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="17" t="n">
+      <c r="Q2" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="17" t="n">
+      <c r="R2" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="17" t="n"/>
+      <c r="S2" s="22" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -693,61 +693,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="15" t="n">
+      <c r="C3" s="19" t="n"/>
+      <c r="D3" s="20" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="17" t="n">
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="22" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="17" t="n">
+      <c r="G3" s="22" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="17" t="n">
+      <c r="H3" s="22" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="17" t="n">
+      <c r="I3" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="17" t="n">
+      <c r="J3" s="22" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="17" t="n">
+      <c r="K3" s="22" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="17" t="n">
+      <c r="L3" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="17" t="n">
+      <c r="M3" s="22" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="17" t="n">
+      <c r="N3" s="22" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="17" t="n">
+      <c r="O3" s="22" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="17" t="n">
+      <c r="P3" s="22" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="17" t="n">
+      <c r="Q3" s="22" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="17" t="n">
+      <c r="R3" s="22" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="17" t="n"/>
+      <c r="S3" s="22" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -755,61 +755,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="15" t="n">
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="20" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="17" t="n">
+      <c r="F4" s="22" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="17" t="n">
+      <c r="G4" s="22" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="17" t="n">
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="17" t="n">
+      <c r="J4" s="22" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="17" t="n">
+      <c r="K4" s="22" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="17" t="n">
+      <c r="L4" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="17" t="n">
+      <c r="M4" s="22" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="17" t="n">
+      <c r="N4" s="22" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="17" t="n">
+      <c r="O4" s="22" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="17" t="n">
+      <c r="P4" s="22" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="17" t="n">
+      <c r="Q4" s="22" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="17" t="n">
+      <c r="R4" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="17" t="n"/>
+      <c r="S4" s="22" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -817,59 +817,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="15" t="n">
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="20" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="22" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="22" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="22" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="I5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="17" t="n">
+      <c r="J5" s="22" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="17" t="n">
+      <c r="K5" s="22" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n">
+      <c r="L5" s="22" t="n"/>
+      <c r="M5" s="22" t="n"/>
+      <c r="N5" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="17" t="n">
+      <c r="O5" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="17" t="n">
+      <c r="P5" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="17" t="n">
+      <c r="Q5" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="17" t="n">
+      <c r="R5" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="17" t="n"/>
+      <c r="S5" s="22" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -877,53 +877,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="15" t="n">
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="20" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="21" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="22" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n">
+      <c r="G6" s="22" t="n"/>
+      <c r="H6" s="22" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="I6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="17" t="n">
+      <c r="J6" s="22" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="K6" s="22" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="17" t="n">
+      <c r="L6" s="22" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n">
+      <c r="M6" s="22" t="n"/>
+      <c r="N6" s="22" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="17" t="n">
+      <c r="O6" s="22" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
-      <c r="S6" s="17" t="n"/>
+      <c r="P6" s="22" t="n"/>
+      <c r="Q6" s="22" t="n"/>
+      <c r="R6" s="22" t="n"/>
+      <c r="S6" s="22" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -931,45 +931,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="15" t="n">
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="20" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="21" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n">
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="22" t="n"/>
+      <c r="H7" s="22" t="n"/>
+      <c r="I7" s="22" t="n"/>
+      <c r="J7" s="22" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="22" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n">
+      <c r="L7" s="22" t="n"/>
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="22" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="17" t="n">
+      <c r="O7" s="22" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
-      <c r="S7" s="17" t="n"/>
+      <c r="P7" s="22" t="n"/>
+      <c r="Q7" s="22" t="n"/>
+      <c r="R7" s="22" t="n"/>
+      <c r="S7" s="22" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -977,367 +977,367 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="15" t="n">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="20" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="21" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="22" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="22" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="17" t="n">
+      <c r="H8" s="22" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="22" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="17" t="n">
+      <c r="K8" s="22" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="17" t="n">
+      <c r="L8" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="17" t="n">
+      <c r="M8" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="17" t="n">
+      <c r="N8" s="22" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="17" t="n">
+      <c r="O8" s="22" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="17" t="n">
+      <c r="P8" s="22" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="17" t="n">
+      <c r="Q8" s="22" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="17" t="n"/>
-      <c r="S8" s="17" t="n"/>
+      <c r="R8" s="22" t="n"/>
+      <c r="S8" s="22" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
-          <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, confirmar. Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos.</t>
+          <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, . Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos. TPV mensual (confirmado por el usuario).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="15" t="n">
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="20" t="n">
         <v>40000000</v>
       </c>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="17" t="n">
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22" t="n">
         <v>0.29</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="22" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="22" t="n">
         <v>0.08</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" s="17" t="n">
+      <c r="J9" s="22" t="n">
         <v>0.0115</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="22" t="n">
         <v>0.0167</v>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="L9" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="M9" s="17" t="n">
+      <c r="M9" s="22" t="n">
         <v>0.025</v>
       </c>
-      <c r="N9" s="17" t="n">
+      <c r="N9" s="22" t="n">
         <v>0.032</v>
       </c>
-      <c r="O9" s="17" t="n">
+      <c r="O9" s="22" t="n">
         <v>0.048</v>
       </c>
-      <c r="P9" s="17" t="n">
+      <c r="P9" s="22" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q9" s="17" t="n">
+      <c r="Q9" s="22" t="n">
         <v>0.105</v>
       </c>
-      <c r="R9" s="17" t="n">
+      <c r="R9" s="22" t="n">
         <v>0.16</v>
       </c>
-      <c r="S9" s="17" t="n"/>
+      <c r="S9" s="22" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (encabezado 'Anual', confirmar base). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
+          <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (mensual, confirmado por el usuario). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n">
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="20" t="n">
         <v>40000000</v>
       </c>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="17" t="n">
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="22" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="22" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="I10" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" s="17" t="n">
+      <c r="J10" s="22" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K10" s="22" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n">
+      <c r="L10" s="22" t="n"/>
+      <c r="M10" s="22" t="n"/>
+      <c r="N10" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O10" s="17" t="n">
+      <c r="O10" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P10" s="17" t="n">
+      <c r="P10" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q10" s="17" t="n">
+      <c r="Q10" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R10" s="17" t="n">
+      <c r="R10" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S10" s="17" t="n"/>
+      <c r="S10" s="22" t="n"/>
       <c r="T10" s="7" t="inlineStr">
         <is>
-          <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece.</t>
+          <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece. TPV mensual (confirmado por el usuario).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="15" t="n">
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="20" t="n">
         <v>136100110.57</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="22" t="n">
         <v>0.6713</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="22" t="n">
         <v>0.3075</v>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="22" t="n">
         <v>0.0212</v>
       </c>
-      <c r="J11" s="17" t="n">
+      <c r="J11" s="22" t="n">
         <v>0.0145</v>
       </c>
-      <c r="K11" s="17" t="n">
+      <c r="K11" s="22" t="n">
         <v>0.018</v>
       </c>
-      <c r="L11" s="17" t="n">
+      <c r="L11" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="M11" s="17" t="n">
+      <c r="M11" s="22" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N11" s="17" t="n">
+      <c r="N11" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O11" s="17" t="n">
+      <c r="O11" s="22" t="n">
         <v>0.075</v>
       </c>
-      <c r="P11" s="17" t="n">
+      <c r="P11" s="22" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q11" s="17" t="n">
+      <c r="Q11" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="R11" s="17" t="n">
+      <c r="R11" s="22" t="n">
         <v>0.18</v>
       </c>
-      <c r="S11" s="17" t="n"/>
+      <c r="S11" s="22" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Origen: 'Monetizacion 0.45%' (encabezado 'ANUAL'). TPV = B3 (anual). Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
+          <t>Origen: 'Monetizacion 0.45%' (mensual, confirmado por el usuario). TPV mensual, confirmado por el usuario. Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n">
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="20" t="n">
         <v>94010839.39</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="22" t="n">
         <v>0.6605</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="22" t="n">
         <v>0.3389</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="I12" s="22" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="J12" s="17" t="n">
+      <c r="J12" s="22" t="n">
         <v>0.0144</v>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K12" s="22" t="n">
         <v>0.0179</v>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n">
+      <c r="L12" s="22" t="n"/>
+      <c r="M12" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" s="17" t="n">
+      <c r="N12" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O12" s="17" t="n">
+      <c r="O12" s="22" t="n">
         <v>0.045</v>
       </c>
-      <c r="P12" s="17" t="n">
+      <c r="P12" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q12" s="17" t="n">
+      <c r="Q12" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R12" s="17" t="n">
+      <c r="R12" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S12" s="17" t="n"/>
+      <c r="S12" s="22" t="n"/>
       <c r="T12" s="7" t="inlineStr">
         <is>
-          <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV = B4. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
+          <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV mensual, confirmado por el usuario. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Caso 3 soluciones</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="15" t="n">
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="20" t="n">
         <v>10000000</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="22" t="n">
         <v>0.28</v>
       </c>
-      <c r="H13" s="17" t="n">
+      <c r="H13" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="I13" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="J13" s="17" t="n">
+      <c r="J13" s="22" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K13" s="17" t="n">
+      <c r="K13" s="22" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L13" s="17" t="n">
+      <c r="L13" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="M13" s="17" t="n">
+      <c r="M13" s="22" t="n">
         <v>0.034</v>
       </c>
-      <c r="N13" s="17" t="n">
+      <c r="N13" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O13" s="17" t="n">
+      <c r="O13" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P13" s="17" t="n">
+      <c r="P13" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="17" t="n">
+      <c r="Q13" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R13" s="17" t="n">
+      <c r="R13" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S13" s="17" t="n"/>
+      <c r="S13" s="22" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
@@ -1345,63 +1345,63 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="15" t="n">
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="20" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G14" s="22" t="n">
         <v>0.24</v>
       </c>
-      <c r="H14" s="17" t="n">
+      <c r="H14" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="17" t="n">
+      <c r="I14" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="J14" s="17" t="n">
+      <c r="J14" s="22" t="n">
         <v>0.0125</v>
       </c>
-      <c r="K14" s="17" t="n">
+      <c r="K14" s="22" t="n">
         <v>0.0161</v>
       </c>
-      <c r="L14" s="17" t="n">
+      <c r="L14" s="22" t="n">
         <v>0.032</v>
       </c>
-      <c r="M14" s="17" t="n">
+      <c r="M14" s="22" t="n">
         <v>0.033</v>
       </c>
-      <c r="N14" s="17" t="n">
+      <c r="N14" s="22" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O14" s="17" t="n">
+      <c r="O14" s="22" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P14" s="17" t="n">
+      <c r="P14" s="22" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q14" s="17" t="n">
+      <c r="Q14" s="22" t="n">
         <v>0.12</v>
       </c>
-      <c r="R14" s="17" t="n">
+      <c r="R14" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S14" s="17" t="n"/>
+      <c r="S14" s="22" t="n"/>
       <c r="T14" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo'. Merchant = CITI. TPV = B3 = B2/12 x C2 (B2 anual 295,435,191 / 12 x 100%). Shares TD B7, TC B8, Int B14. Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. 24x no aparece. Otras hojas: 'EscenarioPsycho' tiene TPV 32M y AMEX/Int distintos (2.6%/2.4%) y 3x 1.91%; 'Flujo Comp (2)' y '1.77-1.99' tienen tasas distintas.</t>
@@ -1409,59 +1409,59 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="15" t="n">
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E15" s="16" t="n">
+      <c r="E15" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="22" t="n">
         <v>0.24</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="H15" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="17" t="n">
+      <c r="I15" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="J15" s="17" t="n">
+      <c r="J15" s="22" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="K15" s="22" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L15" s="17" t="n"/>
-      <c r="M15" s="17" t="n"/>
-      <c r="N15" s="17" t="n">
+      <c r="L15" s="22" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O15" s="17" t="n">
+      <c r="O15" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P15" s="17" t="n">
+      <c r="P15" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q15" s="17" t="n">
+      <c r="Q15" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R15" s="17" t="n">
+      <c r="R15" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S15" s="17" t="n"/>
+      <c r="S15" s="22" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo', sección Fiserv. Mismo TPV y shares que BBVA. Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1469,63 +1469,63 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="15" t="n">
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="20" t="n">
         <v>5200000</v>
       </c>
-      <c r="E16" s="16" t="n">
+      <c r="E16" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="22" t="n">
         <v>0.2</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="22" t="n">
         <v>0.25</v>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="H16" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="17" t="n">
+      <c r="I16" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="17" t="n">
+      <c r="J16" s="22" t="n">
         <v>0.0175</v>
       </c>
-      <c r="K16" s="17" t="n">
+      <c r="K16" s="22" t="n">
         <v>0.0238</v>
       </c>
-      <c r="L16" s="17" t="n">
+      <c r="L16" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="M16" s="17" t="n">
+      <c r="M16" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="N16" s="17" t="n">
+      <c r="N16" s="22" t="n">
         <v>0.0553</v>
       </c>
-      <c r="O16" s="17" t="n">
+      <c r="O16" s="22" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P16" s="17" t="n">
+      <c r="P16" s="22" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q16" s="17" t="n">
+      <c r="Q16" s="22" t="n">
         <v>0.12</v>
       </c>
-      <c r="R16" s="17" t="n">
+      <c r="R16" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S16" s="17" t="n"/>
+      <c r="S16" s="22" t="n"/>
       <c r="T16" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ' (con espacio). TPV = B2 (8M) x C3 (65%). Share TD B7, TC B8 (BBVA MSI 10%, B9, sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI K26:K30. 24x no aparece. Sin periodo en el archivo (confirmar).</t>
@@ -1533,59 +1533,59 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Banamex</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="15" t="n">
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="20" t="n">
         <v>2800000</v>
       </c>
-      <c r="E17" s="16" t="n">
+      <c r="E17" s="21" t="n">
         <v>555</v>
       </c>
-      <c r="F17" s="17" t="n">
+      <c r="F17" s="22" t="n">
         <v>0.2</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="22" t="n">
         <v>0.25</v>
       </c>
-      <c r="H17" s="17" t="n">
+      <c r="H17" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="17" t="n">
+      <c r="I17" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="17" t="n">
+      <c r="J17" s="22" t="n">
         <v>0.018</v>
       </c>
-      <c r="K17" s="17" t="n">
+      <c r="K17" s="22" t="n">
         <v>0.022</v>
       </c>
-      <c r="L17" s="17" t="n"/>
-      <c r="M17" s="17" t="n"/>
-      <c r="N17" s="17" t="n">
+      <c r="L17" s="22" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="22" t="n">
         <v>0.035</v>
       </c>
-      <c r="O17" s="17" t="n">
+      <c r="O17" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="P17" s="17" t="n">
+      <c r="P17" s="22" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q17" s="17" t="n">
+      <c r="Q17" s="22" t="n">
         <v>0.095</v>
       </c>
-      <c r="R17" s="17" t="n">
+      <c r="R17" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="S17" s="17" t="n"/>
+      <c r="S17" s="22" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ', sección Banamex. TPV = B2 (8M) x C4 (35%). Share DEB Banamex B10 (TD), CRE B11 (TC). Débito B38, Crédito B39. Sobretasas MSI K39:K43. Sin AMEX/Internacional. 24x no aparece.</t>

</xml_diff>

<commit_message>
Add ARIAT, Petrolab, Reina Diaz and JULIO CEPEDA competitor rows
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -509,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1888,6 +1903,254 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>ARIAT</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="25" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E23" s="26" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G23" s="27" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H23" s="27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I23" s="27" t="n"/>
+      <c r="J23" s="27" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="K23" s="27" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="L23" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M23" s="27" t="n"/>
+      <c r="N23" s="27" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O23" s="27" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P23" s="27" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q23" s="27" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R23" s="27" t="n"/>
+      <c r="S23" s="27" t="n"/>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja '24h'. Competidor no nombrado ('Solución actual'). TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 1% B8 sin columna). Débito B17, Crédito B18, AMEX B19. Sobretasas MSI K17:K21. Sin Internacional, 18x ni 24x. Suma de shares = 101%. OP (TPV 400k) no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Petrolab</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="25" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="E24" s="26" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G24" s="27" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H24" s="27" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I24" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="27" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="K24" s="27" t="n">
+        <v>0.0218</v>
+      </c>
+      <c r="L24" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M24" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N24" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O24" s="27" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="P24" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q24" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R24" s="27" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="S24" s="27" t="n"/>
+      <c r="T24" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Hoja1'. Competidor no nombrado ('Solución actual'). TPV = B2 ('Procesamiento'), ticket = B3. Shares TD B5, TC B6, AMEX B7, Int = Débito B8 + Crédito B9 (0%). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%). Sobretasas MSI J17:J22. 24x no aparece. OP (TPV 100k) no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Reina Diaz</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="25" t="n">
+        <v>800000</v>
+      </c>
+      <c r="E25" s="26" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G25" s="27" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H25" s="27" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="27" t="n">
+        <v>0.0169</v>
+      </c>
+      <c r="K25" s="27" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="L25" s="27" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="M25" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N25" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O25" s="27" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P25" s="27" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q25" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="R25" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S25" s="27" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Escenario (3)'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int 0 (B8, B9); MSI 10% (B10) sin columna. Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%). Sobretasas MSI J17:J22. 24x no aparece. Escenario (2) y (1) no revisados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>JULIO CEPEDA</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="25" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E26" s="26" t="n">
+        <v>700</v>
+      </c>
+      <c r="F26" s="27" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G26" s="27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I26" s="27" t="n"/>
+      <c r="J26" s="27" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="K26" s="27" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="L26" s="27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M26" s="27" t="n"/>
+      <c r="N26" s="27" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O26" s="27" t="n">
+        <v>0.0395</v>
+      </c>
+      <c r="P26" s="27" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q26" s="27" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="R26" s="27" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="S26" s="27" t="n"/>
+      <c r="T26" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Sin MSIs'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B6, TC B7, AMEX B8 (MSI 3% B9 sin columna). Débito B13, Crédito B14, AMEX B15. Sobretasas MSI K13:K17 (3x con Citi 3.2%, 3x 3.95%). Sin Internacional, 18x ni 24x. Suma de shares = 86%. Hoja 'MSIs' no revisada.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 2CAP, Dega, dENTISTA and APEC competitor rows
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -524,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -652,55 +667,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="19" t="n"/>
-      <c r="D2" s="20" t="n">
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="21" t="n"/>
-      <c r="F2" s="22" t="n">
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="22" t="n">
+      <c r="G2" s="27" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="22" t="n">
+      <c r="H2" s="27" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="22" t="n">
+      <c r="I2" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="22" t="n">
+      <c r="J2" s="27" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="22" t="n"/>
-      <c r="L2" s="22" t="n"/>
-      <c r="M2" s="22" t="n"/>
-      <c r="N2" s="22" t="n">
+      <c r="K2" s="27" t="n"/>
+      <c r="L2" s="27" t="n"/>
+      <c r="M2" s="27" t="n"/>
+      <c r="N2" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="22" t="n">
+      <c r="O2" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="22" t="n">
+      <c r="P2" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="22" t="n">
+      <c r="Q2" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="22" t="n">
+      <c r="R2" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="22" t="n"/>
+      <c r="S2" s="27" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -708,61 +723,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="20" t="n">
+      <c r="C3" s="24" t="n"/>
+      <c r="D3" s="25" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="21" t="n"/>
-      <c r="F3" s="22" t="n">
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="22" t="n">
+      <c r="G3" s="27" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="22" t="n">
+      <c r="H3" s="27" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="27" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="27" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="22" t="n">
+      <c r="L3" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="22" t="n">
+      <c r="M3" s="27" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="27" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="27" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="27" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="27" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="27" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="22" t="n"/>
+      <c r="S3" s="27" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -770,61 +785,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="20" t="n">
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="25" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="E4" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="22" t="n">
+      <c r="F4" s="27" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="22" t="n">
+      <c r="G4" s="27" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="22" t="n"/>
-      <c r="I4" s="22" t="n">
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="27" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="27" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="22" t="n">
+      <c r="L4" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="22" t="n">
+      <c r="M4" s="27" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="22" t="n">
+      <c r="N4" s="27" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="22" t="n">
+      <c r="O4" s="27" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="22" t="n">
+      <c r="P4" s="27" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="22" t="n">
+      <c r="Q4" s="27" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="22" t="n">
+      <c r="R4" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="22" t="n"/>
+      <c r="S4" s="27" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -832,59 +847,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="19" t="n"/>
-      <c r="D5" s="20" t="n">
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="25" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="22" t="n">
+      <c r="F5" s="27" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="27" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="27" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="27" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="27" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="22" t="n"/>
-      <c r="M5" s="22" t="n"/>
-      <c r="N5" s="22" t="n">
+      <c r="L5" s="27" t="n"/>
+      <c r="M5" s="27" t="n"/>
+      <c r="N5" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="22" t="n">
+      <c r="O5" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="22" t="n">
+      <c r="P5" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="22" t="n">
+      <c r="Q5" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="22" t="n">
+      <c r="R5" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="22" t="n"/>
+      <c r="S5" s="27" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -892,53 +907,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="20" t="n">
+      <c r="C6" s="24" t="n"/>
+      <c r="D6" s="25" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="26" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="27" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="22" t="n"/>
-      <c r="H6" s="22" t="n">
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="27" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="27" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="K6" s="27" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="22" t="n">
+      <c r="L6" s="27" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="22" t="n"/>
-      <c r="N6" s="22" t="n">
+      <c r="M6" s="27" t="n"/>
+      <c r="N6" s="27" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="22" t="n">
+      <c r="O6" s="27" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="22" t="n"/>
-      <c r="R6" s="22" t="n"/>
-      <c r="S6" s="22" t="n"/>
+      <c r="P6" s="27" t="n"/>
+      <c r="Q6" s="27" t="n"/>
+      <c r="R6" s="27" t="n"/>
+      <c r="S6" s="27" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -946,45 +961,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="20" t="n">
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="25" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="26" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n">
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="27" t="n"/>
+      <c r="I7" s="27" t="n"/>
+      <c r="J7" s="27" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="K7" s="27" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n">
+      <c r="L7" s="27" t="n"/>
+      <c r="M7" s="27" t="n"/>
+      <c r="N7" s="27" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="22" t="n">
+      <c r="O7" s="27" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
+      <c r="P7" s="27" t="n"/>
+      <c r="Q7" s="27" t="n"/>
+      <c r="R7" s="27" t="n"/>
+      <c r="S7" s="27" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -992,57 +1007,57 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="20" t="n">
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="25" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="26" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="27" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="27" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="22" t="n">
+      <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="27" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="K8" s="27" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="22" t="n">
+      <c r="L8" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="22" t="n">
+      <c r="M8" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="22" t="n">
+      <c r="N8" s="27" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="22" t="n">
+      <c r="O8" s="27" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="22" t="n">
+      <c r="P8" s="27" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="22" t="n">
+      <c r="Q8" s="27" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
+      <c r="R8" s="27" t="n"/>
+      <c r="S8" s="27" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, . Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos. TPV mensual (confirmado por el usuario).</t>
@@ -1050,61 +1065,61 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="20" t="n">
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="25" t="n">
         <v>40000000</v>
       </c>
-      <c r="E9" s="21" t="n"/>
-      <c r="F9" s="22" t="n">
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="27" t="n">
         <v>0.29</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="27" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I9" s="22" t="n">
+      <c r="I9" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="J9" s="27" t="n">
         <v>0.0115</v>
       </c>
-      <c r="K9" s="22" t="n">
+      <c r="K9" s="27" t="n">
         <v>0.0167</v>
       </c>
-      <c r="L9" s="22" t="n">
+      <c r="L9" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="M9" s="22" t="n">
+      <c r="M9" s="27" t="n">
         <v>0.025</v>
       </c>
-      <c r="N9" s="22" t="n">
+      <c r="N9" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="O9" s="22" t="n">
+      <c r="O9" s="27" t="n">
         <v>0.048</v>
       </c>
-      <c r="P9" s="22" t="n">
+      <c r="P9" s="27" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q9" s="22" t="n">
+      <c r="Q9" s="27" t="n">
         <v>0.105</v>
       </c>
-      <c r="R9" s="22" t="n">
+      <c r="R9" s="27" t="n">
         <v>0.16</v>
       </c>
-      <c r="S9" s="22" t="n"/>
+      <c r="S9" s="27" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (mensual, confirmado por el usuario). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
@@ -1112,57 +1127,57 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="20" t="n">
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="25" t="n">
         <v>40000000</v>
       </c>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="22" t="n">
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="27" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" s="22" t="n">
+      <c r="G10" s="27" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="27" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K10" s="22" t="n">
+      <c r="K10" s="27" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L10" s="22" t="n"/>
-      <c r="M10" s="22" t="n"/>
-      <c r="N10" s="22" t="n">
+      <c r="L10" s="27" t="n"/>
+      <c r="M10" s="27" t="n"/>
+      <c r="N10" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O10" s="22" t="n">
+      <c r="O10" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P10" s="22" t="n">
+      <c r="P10" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q10" s="22" t="n">
+      <c r="Q10" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R10" s="22" t="n">
+      <c r="R10" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S10" s="22" t="n"/>
+      <c r="S10" s="27" t="n"/>
       <c r="T10" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece. TPV mensual (confirmado por el usuario).</t>
@@ -1170,63 +1185,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="20" t="n">
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="25" t="n">
         <v>136100110.57</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F11" s="27" t="n">
         <v>0.6713</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G11" s="27" t="n">
         <v>0.3075</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="22" t="n">
+      <c r="I11" s="27" t="n">
         <v>0.0212</v>
       </c>
-      <c r="J11" s="22" t="n">
+      <c r="J11" s="27" t="n">
         <v>0.0145</v>
       </c>
-      <c r="K11" s="22" t="n">
+      <c r="K11" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="L11" s="22" t="n">
+      <c r="L11" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="M11" s="22" t="n">
+      <c r="M11" s="27" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N11" s="22" t="n">
+      <c r="N11" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O11" s="22" t="n">
+      <c r="O11" s="27" t="n">
         <v>0.075</v>
       </c>
-      <c r="P11" s="22" t="n">
+      <c r="P11" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q11" s="22" t="n">
+      <c r="Q11" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="R11" s="22" t="n">
+      <c r="R11" s="27" t="n">
         <v>0.18</v>
       </c>
-      <c r="S11" s="22" t="n"/>
+      <c r="S11" s="27" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%' (mensual, confirmado por el usuario). TPV mensual, confirmado por el usuario. Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
@@ -1234,61 +1249,61 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="20" t="n">
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="25" t="n">
         <v>94010839.39</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="27" t="n">
         <v>0.6605</v>
       </c>
-      <c r="G12" s="22" t="n">
+      <c r="G12" s="27" t="n">
         <v>0.3389</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="H12" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="22" t="n">
+      <c r="I12" s="27" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="J12" s="27" t="n">
         <v>0.0144</v>
       </c>
-      <c r="K12" s="22" t="n">
+      <c r="K12" s="27" t="n">
         <v>0.0179</v>
       </c>
-      <c r="L12" s="22" t="n"/>
-      <c r="M12" s="22" t="n">
+      <c r="L12" s="27" t="n"/>
+      <c r="M12" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" s="22" t="n">
+      <c r="N12" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O12" s="22" t="n">
+      <c r="O12" s="27" t="n">
         <v>0.045</v>
       </c>
-      <c r="P12" s="22" t="n">
+      <c r="P12" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q12" s="22" t="n">
+      <c r="Q12" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R12" s="22" t="n">
+      <c r="R12" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S12" s="22" t="n"/>
+      <c r="S12" s="27" t="n"/>
       <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV mensual, confirmado por el usuario. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
@@ -1296,63 +1311,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Caso 3 soluciones</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="20" t="n">
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="25" t="n">
         <v>10000000</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="22" t="n">
+      <c r="G13" s="27" t="n">
         <v>0.28</v>
       </c>
-      <c r="H13" s="22" t="n">
+      <c r="H13" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="I13" s="22" t="n">
+      <c r="I13" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J13" s="22" t="n">
+      <c r="J13" s="27" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K13" s="22" t="n">
+      <c r="K13" s="27" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L13" s="22" t="n">
+      <c r="L13" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M13" s="22" t="n">
+      <c r="M13" s="27" t="n">
         <v>0.034</v>
       </c>
-      <c r="N13" s="22" t="n">
+      <c r="N13" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O13" s="22" t="n">
+      <c r="O13" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P13" s="22" t="n">
+      <c r="P13" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="22" t="n">
+      <c r="Q13" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R13" s="22" t="n">
+      <c r="R13" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S13" s="22" t="n"/>
+      <c r="S13" s="27" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
@@ -1360,63 +1375,63 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="20" t="n">
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="25" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="27" t="n">
         <v>0.75</v>
       </c>
-      <c r="G14" s="22" t="n">
+      <c r="G14" s="27" t="n">
         <v>0.24</v>
       </c>
-      <c r="H14" s="22" t="n">
+      <c r="H14" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="I14" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="J14" s="27" t="n">
         <v>0.0125</v>
       </c>
-      <c r="K14" s="22" t="n">
+      <c r="K14" s="27" t="n">
         <v>0.0161</v>
       </c>
-      <c r="L14" s="22" t="n">
+      <c r="L14" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="M14" s="22" t="n">
+      <c r="M14" s="27" t="n">
         <v>0.033</v>
       </c>
-      <c r="N14" s="22" t="n">
+      <c r="N14" s="27" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O14" s="22" t="n">
+      <c r="O14" s="27" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P14" s="22" t="n">
+      <c r="P14" s="27" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q14" s="22" t="n">
+      <c r="Q14" s="27" t="n">
         <v>0.12</v>
       </c>
-      <c r="R14" s="22" t="n">
+      <c r="R14" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S14" s="22" t="n"/>
+      <c r="S14" s="27" t="n"/>
       <c r="T14" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo'. Merchant = CITI. TPV = B3 = B2/12 x C2 (B2 anual 295,435,191 / 12 x 100%). Shares TD B7, TC B8, Int B14. Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. 24x no aparece. Otras hojas: 'EscenarioPsycho' tiene TPV 32M y AMEX/Int distintos (2.6%/2.4%) y 3x 1.91%; 'Flujo Comp (2)' y '1.77-1.99' tienen tasas distintas.</t>
@@ -1424,59 +1439,59 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="20" t="n">
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="25" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="27" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="22" t="n">
+      <c r="G15" s="27" t="n">
         <v>0.24</v>
       </c>
-      <c r="H15" s="22" t="n">
+      <c r="H15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="I15" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J15" s="22" t="n">
+      <c r="J15" s="27" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K15" s="22" t="n">
+      <c r="K15" s="27" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L15" s="22" t="n"/>
-      <c r="M15" s="22" t="n"/>
-      <c r="N15" s="22" t="n">
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="27" t="n"/>
+      <c r="N15" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O15" s="22" t="n">
+      <c r="O15" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P15" s="22" t="n">
+      <c r="P15" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q15" s="22" t="n">
+      <c r="Q15" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R15" s="22" t="n">
+      <c r="R15" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S15" s="22" t="n"/>
+      <c r="S15" s="27" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo', sección Fiserv. Mismo TPV y shares que BBVA. Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1484,63 +1499,63 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="23" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="20" t="n">
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="25" t="n">
         <v>5200000</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F16" s="22" t="n">
+      <c r="F16" s="27" t="n">
         <v>0.2</v>
       </c>
-      <c r="G16" s="22" t="n">
+      <c r="G16" s="27" t="n">
         <v>0.25</v>
       </c>
-      <c r="H16" s="22" t="n">
+      <c r="H16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="I16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="22" t="n">
+      <c r="J16" s="27" t="n">
         <v>0.0175</v>
       </c>
-      <c r="K16" s="22" t="n">
+      <c r="K16" s="27" t="n">
         <v>0.0238</v>
       </c>
-      <c r="L16" s="22" t="n">
+      <c r="L16" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="M16" s="22" t="n">
+      <c r="M16" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="N16" s="22" t="n">
+      <c r="N16" s="27" t="n">
         <v>0.0553</v>
       </c>
-      <c r="O16" s="22" t="n">
+      <c r="O16" s="27" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P16" s="22" t="n">
+      <c r="P16" s="27" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q16" s="22" t="n">
+      <c r="Q16" s="27" t="n">
         <v>0.12</v>
       </c>
-      <c r="R16" s="22" t="n">
+      <c r="R16" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S16" s="22" t="n"/>
+      <c r="S16" s="27" t="n"/>
       <c r="T16" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ' (con espacio). TPV = B2 (8M) x C3 (65%). Share TD B7, TC B8 (BBVA MSI 10%, B9, sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI K26:K30. 24x no aparece. Sin periodo en el archivo (confirmar).</t>
@@ -1548,59 +1563,59 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="23" t="inlineStr">
         <is>
           <t>Banamex</t>
         </is>
       </c>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="20" t="n">
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="25" t="n">
         <v>2800000</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="26" t="n">
         <v>555</v>
       </c>
-      <c r="F17" s="22" t="n">
+      <c r="F17" s="27" t="n">
         <v>0.2</v>
       </c>
-      <c r="G17" s="22" t="n">
+      <c r="G17" s="27" t="n">
         <v>0.25</v>
       </c>
-      <c r="H17" s="22" t="n">
+      <c r="H17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="22" t="n">
+      <c r="I17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="22" t="n">
+      <c r="J17" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="K17" s="22" t="n">
+      <c r="K17" s="27" t="n">
         <v>0.022</v>
       </c>
-      <c r="L17" s="22" t="n"/>
-      <c r="M17" s="22" t="n"/>
-      <c r="N17" s="22" t="n">
+      <c r="L17" s="27" t="n"/>
+      <c r="M17" s="27" t="n"/>
+      <c r="N17" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="O17" s="22" t="n">
+      <c r="O17" s="27" t="n">
         <v>0.04</v>
       </c>
-      <c r="P17" s="22" t="n">
+      <c r="P17" s="27" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q17" s="22" t="n">
+      <c r="Q17" s="27" t="n">
         <v>0.095</v>
       </c>
-      <c r="R17" s="22" t="n">
+      <c r="R17" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S17" s="22" t="n"/>
+      <c r="S17" s="27" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ', sección Banamex. TPV = B2 (8M) x C4 (35%). Share DEB Banamex B10 (TD), CRE B11 (TC). Débito B38, Crédito B39. Sobretasas MSI K39:K43. Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1608,57 +1623,57 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Florence</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="23" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="20" t="n">
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="25" t="n">
         <v>4000000</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="26" t="n">
         <v>60000</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G18" s="22" t="n">
+      <c r="G18" s="27" t="n">
         <v>0.49</v>
       </c>
-      <c r="H18" s="22" t="n">
+      <c r="H18" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I18" s="22" t="n"/>
-      <c r="J18" s="22" t="n">
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="K18" s="22" t="n">
+      <c r="K18" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="L18" s="22" t="n">
+      <c r="L18" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="22" t="n">
+      <c r="M18" s="27" t="n"/>
+      <c r="N18" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="O18" s="22" t="n">
+      <c r="O18" s="27" t="n">
         <v>0.055</v>
       </c>
-      <c r="P18" s="22" t="n">
+      <c r="P18" s="27" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q18" s="22" t="n">
+      <c r="Q18" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
+      <c r="R18" s="27" t="n"/>
+      <c r="S18" s="27" t="n"/>
       <c r="T18" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1666,57 +1681,57 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>grupo_milano</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="20" t="n">
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="25" t="n">
         <v>4000000</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="26" t="n">
         <v>60000</v>
       </c>
-      <c r="F19" s="22" t="n">
+      <c r="F19" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G19" s="27" t="n">
         <v>0.49</v>
       </c>
-      <c r="H19" s="22" t="n">
+      <c r="H19" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="22" t="n">
+      <c r="I19" s="27" t="n"/>
+      <c r="J19" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="K19" s="22" t="n">
+      <c r="K19" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="L19" s="22" t="n">
+      <c r="L19" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M19" s="22" t="n"/>
-      <c r="N19" s="22" t="n">
+      <c r="M19" s="27" t="n"/>
+      <c r="N19" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="O19" s="22" t="n">
+      <c r="O19" s="27" t="n">
         <v>0.055</v>
       </c>
-      <c r="P19" s="22" t="n">
+      <c r="P19" s="27" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q19" s="22" t="n">
+      <c r="Q19" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
+      <c r="R19" s="27" t="n"/>
+      <c r="S19" s="27" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1724,57 +1739,57 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>Carlos Toys</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="20" t="n">
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="25" t="n">
         <v>4000000</v>
       </c>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="26" t="n">
         <v>60000</v>
       </c>
-      <c r="F20" s="22" t="n">
+      <c r="F20" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G20" s="22" t="n">
+      <c r="G20" s="27" t="n">
         <v>0.49</v>
       </c>
-      <c r="H20" s="22" t="n">
+      <c r="H20" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I20" s="22" t="n"/>
-      <c r="J20" s="22" t="n">
+      <c r="I20" s="27" t="n"/>
+      <c r="J20" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="K20" s="22" t="n">
+      <c r="K20" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="L20" s="22" t="n">
+      <c r="L20" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M20" s="22" t="n"/>
-      <c r="N20" s="22" t="n">
+      <c r="M20" s="27" t="n"/>
+      <c r="N20" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="O20" s="22" t="n">
+      <c r="O20" s="27" t="n">
         <v>0.055</v>
       </c>
-      <c r="P20" s="22" t="n">
+      <c r="P20" s="27" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q20" s="22" t="n">
+      <c r="Q20" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
+      <c r="R20" s="27" t="n"/>
+      <c r="S20" s="27" t="n"/>
       <c r="T20" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1782,57 +1797,57 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>Kaloni</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="20" t="n">
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="25" t="n">
         <v>4000000</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="26" t="n">
         <v>60000</v>
       </c>
-      <c r="F21" s="22" t="n">
+      <c r="F21" s="27" t="n">
         <v>0.43</v>
       </c>
-      <c r="G21" s="22" t="n">
+      <c r="G21" s="27" t="n">
         <v>0.49</v>
       </c>
-      <c r="H21" s="22" t="n">
+      <c r="H21" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="I21" s="22" t="n"/>
-      <c r="J21" s="22" t="n">
+      <c r="I21" s="27" t="n"/>
+      <c r="J21" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="K21" s="22" t="n">
+      <c r="K21" s="27" t="n">
         <v>0.018</v>
       </c>
-      <c r="L21" s="22" t="n">
+      <c r="L21" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="M21" s="22" t="n"/>
-      <c r="N21" s="22" t="n">
+      <c r="M21" s="27" t="n"/>
+      <c r="N21" s="27" t="n">
         <v>0.032</v>
       </c>
-      <c r="O21" s="22" t="n">
+      <c r="O21" s="27" t="n">
         <v>0.055</v>
       </c>
-      <c r="P21" s="22" t="n">
+      <c r="P21" s="27" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q21" s="22" t="n">
+      <c r="Q21" s="27" t="n">
         <v>0.11</v>
       </c>
-      <c r="R21" s="22" t="n"/>
-      <c r="S21" s="22" t="n"/>
+      <c r="R21" s="27" t="n"/>
+      <c r="S21" s="27" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1840,63 +1855,63 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Bobois</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="20" t="n">
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="25" t="n">
         <v>6000000</v>
       </c>
-      <c r="E22" s="21" t="n">
+      <c r="E22" s="26" t="n">
         <v>800</v>
       </c>
-      <c r="F22" s="22" t="n">
+      <c r="F22" s="27" t="n">
         <v>0.5</v>
       </c>
-      <c r="G22" s="22" t="n">
+      <c r="G22" s="27" t="n">
         <v>0.48</v>
       </c>
-      <c r="H22" s="22" t="n">
+      <c r="H22" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="I22" s="27" t="n">
         <v>0.01</v>
       </c>
-      <c r="J22" s="22" t="n">
+      <c r="J22" s="27" t="n">
         <v>0.015</v>
       </c>
-      <c r="K22" s="22" t="n">
+      <c r="K22" s="27" t="n">
         <v>0.0185</v>
       </c>
-      <c r="L22" s="22" t="n">
+      <c r="L22" s="27" t="n">
         <v>0.029</v>
       </c>
-      <c r="M22" s="22" t="n">
+      <c r="M22" s="27" t="n">
         <v>0.03</v>
       </c>
-      <c r="N22" s="22" t="n">
+      <c r="N22" s="27" t="n">
         <v>0.05</v>
       </c>
-      <c r="O22" s="22" t="n">
+      <c r="O22" s="27" t="n">
         <v>0.05</v>
       </c>
-      <c r="P22" s="22" t="n">
+      <c r="P22" s="27" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q22" s="22" t="n">
+      <c r="Q22" s="27" t="n">
         <v>0.1</v>
       </c>
-      <c r="R22" s="22" t="n">
+      <c r="R22" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="S22" s="22" t="n"/>
+      <c r="S22" s="27" t="n"/>
       <c r="T22" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario 24 horas '. Competidor no nombrado ('Solución actual'). TPV = B2 (6M), ticket = B3. Shares TD B5, TC B6, AMEX B7, Internacional = Débito B8 + Crédito B9 (0.5% + 0.5%). MSI 0% (B10). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%) - ambos 3.0%. Sobretasas MSI K17:K22 (3x con Citi 5% y 3x 5%; 18x 18.9%). 24x no aparece. Otras hojas (Escenario 1, 48 horas, citi 3x, Hoja2) tienen valores distintos.</t>
@@ -2148,6 +2163,376 @@
       <c r="T26" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Sin MSIs'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B6, TC B7, AMEX B8 (MSI 3% B9 sin columna). Débito B13, Crédito B14, AMEX B15. Sobretasas MSI K13:K17 (3x con Citi 3.2%, 3x 3.95%). Sin Internacional, 18x ni 24x. Suma de shares = 86%. Hoja 'MSIs' no revisada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>2CAP (Nacional)</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="30" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="E27" s="31" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F27" s="32" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G27" s="32" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H27" s="32" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I27" s="32" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J27" s="32" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K27" s="32" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="L27" s="32" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M27" s="32" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="N27" s="32" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O27" s="32" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P27" s="32" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="Q27" s="32" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="R27" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S27" s="32" t="n"/>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Monetizacion Aeropuerto T7', bloque 'Procesamiento Actual en terminales' (B2:B11). Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int Débito B8 (MSI 5% B11 sin columna). Débito B24, Crédito B25, AMEX B26, Int B27. Sobretasas MSI J24:J29. 24x no aparece. Otras hojas (T4, T2, 2/4/7 DIAS) no revisadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>2CAP (Aeropuerto T7)</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="30" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="E28" s="31" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F28" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G28" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H28" s="32" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I28" s="32" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J28" s="32" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="K28" s="32" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="L28" s="32" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M28" s="32" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="N28" s="32" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O28" s="32" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P28" s="32" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="Q28" s="32" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="R28" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S28" s="32" t="n"/>
+      <c r="T28" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Monetizacion Aeropuerto T7', bloque 'Procesamiento Actual en Aeropuertos' (D2:E9). TPV = E2, ticket = E3. Shares TD E5, TC E6, AMEX E7, Int Débito E8 = 70% (revisar, parece alto). Tasas B36:B39 y sobretasas J36:J41 iguales al nacional. 24x no aparece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>Dega</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="30" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E29" s="31" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F29" s="32" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="G29" s="32" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="H29" s="32" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I29" s="32" t="n"/>
+      <c r="J29" s="32" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="K29" s="32" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="L29" s="32" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M29" s="32" t="n"/>
+      <c r="N29" s="32" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O29" s="32" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P29" s="32" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q29" s="32" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="R29" s="32" t="n"/>
+      <c r="S29" s="32" t="n"/>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Hoja1'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 8% B8 sin columna; la suma TD+TC+AMEX+MSI = 108%, revisar). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. OP no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>dENTISTA</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="30" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F30" s="32" t="n">
+        <v>0.3795</v>
+      </c>
+      <c r="G30" s="32" t="n">
+        <v>0.2192</v>
+      </c>
+      <c r="H30" s="32" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="I30" s="32" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J30" s="32" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="K30" s="32" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="L30" s="32" t="n">
+        <v>0.0293</v>
+      </c>
+      <c r="M30" s="32" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="N30" s="32" t="n">
+        <v>0.0485</v>
+      </c>
+      <c r="O30" s="32" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="P30" s="32" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="Q30" s="32" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="R30" s="32" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="S30" s="32" t="n"/>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Hoja1'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int = Débito B8 + Crédito B9 (3.5% + 3.5%). MSI 31% (B10) sin columna. Débito B15, Crédito B16, AMEX B17, Int Crédito B18 (1.4%), Int Débito B19 (1.4%). Sobretasas MSI J15:J20 (3x con Citi = 3x = 4.85%). Sin 24x. Tasa TD/TC (0.9%) muy baja, revisar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>APEC</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>BBVA</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="30" t="n">
+        <v>21780000</v>
+      </c>
+      <c r="E31" s="31" t="n">
+        <v>555</v>
+      </c>
+      <c r="F31" s="32" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="G31" s="32" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H31" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="32" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="J31" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="32" t="n">
+        <v>0.009900000000000001</v>
+      </c>
+      <c r="L31" s="32" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M31" s="32" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="N31" s="32" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O31" s="32" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="P31" s="32" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="Q31" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R31" s="32" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="S31" s="32" t="n"/>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Monetizacion 0.60%'. TPV = B3 (B2 x C3 = 66%). Shares TD B7, TC B8, Int B14 (7%, total). BBVA MSI 10% (B9) sin columna. Débito B25 = 0% (revisar; la tasa base TC aparece como 0.99% en J25:J30), Crédito B26, AMEX B27, Int B28. Sobretasas MSI K25:K30. 24x no aparece. TPV sin periodo (tratado como mensual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>APEC</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Scotia</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="30" t="n">
+        <v>11220000</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <v>555</v>
+      </c>
+      <c r="F32" s="32" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G32" s="32" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H32" s="32" t="n"/>
+      <c r="I32" s="32" t="n"/>
+      <c r="J32" s="32" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="K32" s="32" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="L32" s="32" t="n"/>
+      <c r="M32" s="32" t="n"/>
+      <c r="N32" s="32" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O32" s="32" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="P32" s="32" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q32" s="32" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R32" s="32" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S32" s="32" t="n"/>
+      <c r="T32" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja activa 'Monetizacion 0.60%', sección Scotia (B4 'mifel' = 34%, TPV = B4). Shares DEB SCOTIA B10 (TD), CRE SCOTIA B11 (TC), MSI SCOTIA 22% (B13) sin columna. Débito B38, Crédito B39. Sobretasas MSI K39:K43. 6x = 4.5% (K40); 6x con Citibanamex = 8.76% (K38) no mapeada. Sin AMEX/Internacional. 24x no aparece.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add HI TEK, DHI Clinic, Diagsa, Christus and photo sellers (with Industria)
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -539,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:T41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -667,55 +682,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="24" t="n"/>
-      <c r="D2" s="25" t="n">
+      <c r="C2" s="29" t="n"/>
+      <c r="D2" s="30" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="26" t="n"/>
-      <c r="F2" s="27" t="n">
+      <c r="E2" s="31" t="n"/>
+      <c r="F2" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="27" t="n">
+      <c r="G2" s="32" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="27" t="n">
+      <c r="H2" s="32" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="27" t="n">
+      <c r="I2" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="27" t="n">
+      <c r="J2" s="32" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="27" t="n"/>
-      <c r="L2" s="27" t="n"/>
-      <c r="M2" s="27" t="n"/>
-      <c r="N2" s="27" t="n">
+      <c r="K2" s="32" t="n"/>
+      <c r="L2" s="32" t="n"/>
+      <c r="M2" s="32" t="n"/>
+      <c r="N2" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="27" t="n">
+      <c r="O2" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="27" t="n">
+      <c r="P2" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="27" t="n">
+      <c r="Q2" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="27" t="n">
+      <c r="R2" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="27" t="n"/>
+      <c r="S2" s="32" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -723,61 +738,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="24" t="n"/>
-      <c r="D3" s="25" t="n">
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="30" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="26" t="n"/>
-      <c r="F3" s="27" t="n">
+      <c r="E3" s="31" t="n"/>
+      <c r="F3" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="27" t="n">
+      <c r="G3" s="32" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="27" t="n">
+      <c r="H3" s="32" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="27" t="n">
+      <c r="I3" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="27" t="n">
+      <c r="J3" s="32" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="27" t="n">
+      <c r="K3" s="32" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="27" t="n">
+      <c r="L3" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="32" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="27" t="n">
+      <c r="N3" s="32" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="27" t="n">
+      <c r="O3" s="32" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="27" t="n">
+      <c r="P3" s="32" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="27" t="n">
+      <c r="Q3" s="32" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="27" t="n">
+      <c r="R3" s="32" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="27" t="n"/>
+      <c r="S3" s="32" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -785,61 +800,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="24" t="n"/>
-      <c r="D4" s="25" t="n">
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="30" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="32" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="27" t="n">
+      <c r="G4" s="32" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="27" t="n"/>
-      <c r="I4" s="27" t="n">
+      <c r="H4" s="32" t="n"/>
+      <c r="I4" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="27" t="n">
+      <c r="J4" s="32" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="27" t="n">
+      <c r="K4" s="32" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="27" t="n">
+      <c r="L4" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="32" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="27" t="n">
+      <c r="N4" s="32" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="27" t="n">
+      <c r="O4" s="32" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="27" t="n">
+      <c r="P4" s="32" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="27" t="n">
+      <c r="Q4" s="32" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="27" t="n">
+      <c r="R4" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="27" t="n"/>
+      <c r="S4" s="32" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -847,59 +862,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="25" t="n">
+      <c r="C5" s="29" t="n"/>
+      <c r="D5" s="30" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="32" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="32" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="32" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="27" t="n">
+      <c r="J5" s="32" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="27" t="n">
+      <c r="K5" s="32" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="27" t="n"/>
-      <c r="M5" s="27" t="n"/>
-      <c r="N5" s="27" t="n">
+      <c r="L5" s="32" t="n"/>
+      <c r="M5" s="32" t="n"/>
+      <c r="N5" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="27" t="n">
+      <c r="O5" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="27" t="n">
+      <c r="P5" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="27" t="n">
+      <c r="Q5" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="27" t="n">
+      <c r="R5" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="27" t="n"/>
+      <c r="S5" s="32" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -907,53 +922,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="25" t="n">
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="30" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="31" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="32" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="27" t="n"/>
-      <c r="H6" s="27" t="n">
+      <c r="G6" s="32" t="n"/>
+      <c r="H6" s="32" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="27" t="n">
+      <c r="J6" s="32" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="27" t="n">
+      <c r="K6" s="32" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="32" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="27" t="n"/>
-      <c r="N6" s="27" t="n">
+      <c r="M6" s="32" t="n"/>
+      <c r="N6" s="32" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="27" t="n">
+      <c r="O6" s="32" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="27" t="n"/>
-      <c r="Q6" s="27" t="n"/>
-      <c r="R6" s="27" t="n"/>
-      <c r="S6" s="27" t="n"/>
+      <c r="P6" s="32" t="n"/>
+      <c r="Q6" s="32" t="n"/>
+      <c r="R6" s="32" t="n"/>
+      <c r="S6" s="32" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -961,45 +976,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="25" t="n">
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="30" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="31" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
-      <c r="I7" s="27" t="n"/>
-      <c r="J7" s="27" t="n">
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="n"/>
+      <c r="J7" s="32" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="27" t="n">
+      <c r="K7" s="32" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="27" t="n"/>
-      <c r="M7" s="27" t="n"/>
-      <c r="N7" s="27" t="n">
+      <c r="L7" s="32" t="n"/>
+      <c r="M7" s="32" t="n"/>
+      <c r="N7" s="32" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="27" t="n">
+      <c r="O7" s="32" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="27" t="n"/>
-      <c r="Q7" s="27" t="n"/>
-      <c r="R7" s="27" t="n"/>
-      <c r="S7" s="27" t="n"/>
+      <c r="P7" s="32" t="n"/>
+      <c r="Q7" s="32" t="n"/>
+      <c r="R7" s="32" t="n"/>
+      <c r="S7" s="32" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -1007,57 +1022,57 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="25" t="n">
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="30" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E8" s="31" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="32" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="27" t="n"/>
-      <c r="I8" s="27" t="n"/>
-      <c r="J8" s="27" t="n">
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="n"/>
+      <c r="J8" s="32" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="27" t="n">
+      <c r="K8" s="32" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="27" t="n">
+      <c r="L8" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="27" t="n">
+      <c r="N8" s="32" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="27" t="n">
+      <c r="O8" s="32" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="27" t="n">
+      <c r="P8" s="32" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="27" t="n">
+      <c r="Q8" s="32" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="27" t="n"/>
-      <c r="S8" s="27" t="n"/>
+      <c r="R8" s="32" t="n"/>
+      <c r="S8" s="32" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, . Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos. TPV mensual (confirmado por el usuario).</t>
@@ -1065,61 +1080,61 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="25" t="n">
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="30" t="n">
         <v>40000000</v>
       </c>
-      <c r="E9" s="26" t="n"/>
-      <c r="F9" s="27" t="n">
+      <c r="E9" s="31" t="n"/>
+      <c r="F9" s="32" t="n">
         <v>0.29</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" s="27" t="n">
+      <c r="J9" s="32" t="n">
         <v>0.0115</v>
       </c>
-      <c r="K9" s="27" t="n">
+      <c r="K9" s="32" t="n">
         <v>0.0167</v>
       </c>
-      <c r="L9" s="27" t="n">
+      <c r="L9" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="32" t="n">
         <v>0.025</v>
       </c>
-      <c r="N9" s="27" t="n">
+      <c r="N9" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O9" s="27" t="n">
+      <c r="O9" s="32" t="n">
         <v>0.048</v>
       </c>
-      <c r="P9" s="27" t="n">
+      <c r="P9" s="32" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q9" s="27" t="n">
+      <c r="Q9" s="32" t="n">
         <v>0.105</v>
       </c>
-      <c r="R9" s="27" t="n">
+      <c r="R9" s="32" t="n">
         <v>0.16</v>
       </c>
-      <c r="S9" s="27" t="n"/>
+      <c r="S9" s="32" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (mensual, confirmado por el usuario). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
@@ -1127,57 +1142,57 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="25" t="n">
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="30" t="n">
         <v>40000000</v>
       </c>
-      <c r="E10" s="26" t="n"/>
-      <c r="F10" s="27" t="n">
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="32" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="32" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" s="27" t="n">
+      <c r="H10" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" s="27" t="n">
+      <c r="J10" s="32" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K10" s="27" t="n">
+      <c r="K10" s="32" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L10" s="27" t="n"/>
-      <c r="M10" s="27" t="n"/>
-      <c r="N10" s="27" t="n">
+      <c r="L10" s="32" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O10" s="27" t="n">
+      <c r="O10" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P10" s="27" t="n">
+      <c r="P10" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q10" s="27" t="n">
+      <c r="Q10" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R10" s="27" t="n">
+      <c r="R10" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S10" s="27" t="n"/>
+      <c r="S10" s="32" t="n"/>
       <c r="T10" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece. TPV mensual (confirmado por el usuario).</t>
@@ -1185,63 +1200,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="25" t="n">
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="30" t="n">
         <v>136100110.57</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="32" t="n">
         <v>0.6713</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="32" t="n">
         <v>0.3075</v>
       </c>
-      <c r="H11" s="27" t="n">
+      <c r="H11" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="27" t="n">
+      <c r="I11" s="32" t="n">
         <v>0.0212</v>
       </c>
-      <c r="J11" s="27" t="n">
+      <c r="J11" s="32" t="n">
         <v>0.0145</v>
       </c>
-      <c r="K11" s="27" t="n">
+      <c r="K11" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="L11" s="27" t="n">
+      <c r="L11" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="32" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N11" s="27" t="n">
+      <c r="N11" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O11" s="27" t="n">
+      <c r="O11" s="32" t="n">
         <v>0.075</v>
       </c>
-      <c r="P11" s="27" t="n">
+      <c r="P11" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q11" s="27" t="n">
+      <c r="Q11" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="R11" s="27" t="n">
+      <c r="R11" s="32" t="n">
         <v>0.18</v>
       </c>
-      <c r="S11" s="27" t="n"/>
+      <c r="S11" s="32" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%' (mensual, confirmado por el usuario). TPV mensual, confirmado por el usuario. Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
@@ -1249,61 +1264,61 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="25" t="n">
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="30" t="n">
         <v>94010839.39</v>
       </c>
-      <c r="E12" s="26" t="n">
+      <c r="E12" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="32" t="n">
         <v>0.6605</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="32" t="n">
         <v>0.3389</v>
       </c>
-      <c r="H12" s="27" t="n">
+      <c r="H12" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="32" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="J12" s="27" t="n">
+      <c r="J12" s="32" t="n">
         <v>0.0144</v>
       </c>
-      <c r="K12" s="27" t="n">
+      <c r="K12" s="32" t="n">
         <v>0.0179</v>
       </c>
-      <c r="L12" s="27" t="n"/>
-      <c r="M12" s="27" t="n">
+      <c r="L12" s="32" t="n"/>
+      <c r="M12" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" s="27" t="n">
+      <c r="N12" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O12" s="27" t="n">
+      <c r="O12" s="32" t="n">
         <v>0.045</v>
       </c>
-      <c r="P12" s="27" t="n">
+      <c r="P12" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q12" s="27" t="n">
+      <c r="Q12" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R12" s="27" t="n">
+      <c r="R12" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S12" s="27" t="n"/>
+      <c r="S12" s="32" t="n"/>
       <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV mensual, confirmado por el usuario. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
@@ -1311,63 +1326,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Caso 3 soluciones</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="28" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="25" t="n">
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="30" t="n">
         <v>10000000</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="32" t="n">
         <v>0.28</v>
       </c>
-      <c r="H13" s="27" t="n">
+      <c r="H13" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="I13" s="27" t="n">
+      <c r="I13" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J13" s="27" t="n">
+      <c r="J13" s="32" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K13" s="27" t="n">
+      <c r="K13" s="32" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L13" s="27" t="n">
+      <c r="L13" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="32" t="n">
         <v>0.034</v>
       </c>
-      <c r="N13" s="27" t="n">
+      <c r="N13" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O13" s="27" t="n">
+      <c r="O13" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P13" s="27" t="n">
+      <c r="P13" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="27" t="n">
+      <c r="Q13" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R13" s="27" t="n">
+      <c r="R13" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S13" s="27" t="n"/>
+      <c r="S13" s="32" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
@@ -1375,63 +1390,63 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="25" t="n">
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="30" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E14" s="26" t="n">
+      <c r="E14" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="32" t="n">
         <v>0.75</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="32" t="n">
         <v>0.24</v>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="27" t="n">
+      <c r="I14" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J14" s="27" t="n">
+      <c r="J14" s="32" t="n">
         <v>0.0125</v>
       </c>
-      <c r="K14" s="27" t="n">
+      <c r="K14" s="32" t="n">
         <v>0.0161</v>
       </c>
-      <c r="L14" s="27" t="n">
+      <c r="L14" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="32" t="n">
         <v>0.033</v>
       </c>
-      <c r="N14" s="27" t="n">
+      <c r="N14" s="32" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O14" s="27" t="n">
+      <c r="O14" s="32" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P14" s="27" t="n">
+      <c r="P14" s="32" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q14" s="27" t="n">
+      <c r="Q14" s="32" t="n">
         <v>0.12</v>
       </c>
-      <c r="R14" s="27" t="n">
+      <c r="R14" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S14" s="27" t="n"/>
+      <c r="S14" s="32" t="n"/>
       <c r="T14" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo'. Merchant = CITI. TPV = B3 = B2/12 x C2 (B2 anual 295,435,191 / 12 x 100%). Shares TD B7, TC B8, Int B14. Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. 24x no aparece. Otras hojas: 'EscenarioPsycho' tiene TPV 32M y AMEX/Int distintos (2.6%/2.4%) y 3x 1.91%; 'Flujo Comp (2)' y '1.77-1.99' tienen tasas distintas.</t>
@@ -1439,59 +1454,59 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="25" t="n">
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="30" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="32" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="32" t="n">
         <v>0.24</v>
       </c>
-      <c r="H15" s="27" t="n">
+      <c r="H15" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="27" t="n">
+      <c r="I15" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J15" s="27" t="n">
+      <c r="J15" s="32" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K15" s="27" t="n">
+      <c r="K15" s="32" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L15" s="27" t="n"/>
-      <c r="M15" s="27" t="n"/>
-      <c r="N15" s="27" t="n">
+      <c r="L15" s="32" t="n"/>
+      <c r="M15" s="32" t="n"/>
+      <c r="N15" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O15" s="27" t="n">
+      <c r="O15" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P15" s="27" t="n">
+      <c r="P15" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q15" s="27" t="n">
+      <c r="Q15" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R15" s="27" t="n">
+      <c r="R15" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S15" s="27" t="n"/>
+      <c r="S15" s="32" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo', sección Fiserv. Mismo TPV y shares que BBVA. Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1499,63 +1514,63 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="25" t="n">
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="30" t="n">
         <v>5200000</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E16" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="27" t="n">
+      <c r="J16" s="32" t="n">
         <v>0.0175</v>
       </c>
-      <c r="K16" s="27" t="n">
+      <c r="K16" s="32" t="n">
         <v>0.0238</v>
       </c>
-      <c r="L16" s="27" t="n">
+      <c r="L16" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="M16" s="27" t="n">
+      <c r="M16" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="N16" s="27" t="n">
+      <c r="N16" s="32" t="n">
         <v>0.0553</v>
       </c>
-      <c r="O16" s="27" t="n">
+      <c r="O16" s="32" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P16" s="27" t="n">
+      <c r="P16" s="32" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q16" s="27" t="n">
+      <c r="Q16" s="32" t="n">
         <v>0.12</v>
       </c>
-      <c r="R16" s="27" t="n">
+      <c r="R16" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S16" s="27" t="n"/>
+      <c r="S16" s="32" t="n"/>
       <c r="T16" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ' (con espacio). TPV = B2 (8M) x C3 (65%). Share TD B7, TC B8 (BBVA MSI 10%, B9, sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI K26:K30. 24x no aparece. Sin periodo en el archivo (confirmar).</t>
@@ -1563,59 +1578,59 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Banamex</t>
         </is>
       </c>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="25" t="n">
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="30" t="n">
         <v>2800000</v>
       </c>
-      <c r="E17" s="26" t="n">
+      <c r="E17" s="31" t="n">
         <v>555</v>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F17" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="32" t="n">
         <v>0.25</v>
       </c>
-      <c r="H17" s="27" t="n">
+      <c r="H17" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="27" t="n">
+      <c r="I17" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="27" t="n">
+      <c r="J17" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="K17" s="27" t="n">
+      <c r="K17" s="32" t="n">
         <v>0.022</v>
       </c>
-      <c r="L17" s="27" t="n"/>
-      <c r="M17" s="27" t="n"/>
-      <c r="N17" s="27" t="n">
+      <c r="L17" s="32" t="n"/>
+      <c r="M17" s="32" t="n"/>
+      <c r="N17" s="32" t="n">
         <v>0.035</v>
       </c>
-      <c r="O17" s="27" t="n">
+      <c r="O17" s="32" t="n">
         <v>0.04</v>
       </c>
-      <c r="P17" s="27" t="n">
+      <c r="P17" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q17" s="27" t="n">
+      <c r="Q17" s="32" t="n">
         <v>0.095</v>
       </c>
-      <c r="R17" s="27" t="n">
+      <c r="R17" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S17" s="27" t="n"/>
+      <c r="S17" s="32" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ', sección Banamex. TPV = B2 (8M) x C4 (35%). Share DEB Banamex B10 (TD), CRE B11 (TC). Débito B38, Crédito B39. Sobretasas MSI K39:K43. Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1623,57 +1638,57 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>Florence</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="25" t="n">
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="30" t="n">
         <v>4000000</v>
       </c>
-      <c r="E18" s="26" t="n">
+      <c r="E18" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="32" t="n">
         <v>0.49</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I18" s="27" t="n"/>
-      <c r="J18" s="27" t="n">
+      <c r="I18" s="32" t="n"/>
+      <c r="J18" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="K18" s="27" t="n">
+      <c r="K18" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="L18" s="27" t="n">
+      <c r="L18" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M18" s="27" t="n"/>
-      <c r="N18" s="27" t="n">
+      <c r="M18" s="32" t="n"/>
+      <c r="N18" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O18" s="27" t="n">
+      <c r="O18" s="32" t="n">
         <v>0.055</v>
       </c>
-      <c r="P18" s="27" t="n">
+      <c r="P18" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q18" s="27" t="n">
+      <c r="Q18" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="R18" s="27" t="n"/>
-      <c r="S18" s="27" t="n"/>
+      <c r="R18" s="32" t="n"/>
+      <c r="S18" s="32" t="n"/>
       <c r="T18" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1681,57 +1696,57 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>grupo_milano</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="25" t="n">
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="30" t="n">
         <v>4000000</v>
       </c>
-      <c r="E19" s="26" t="n">
+      <c r="E19" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G19" s="32" t="n">
         <v>0.49</v>
       </c>
-      <c r="H19" s="27" t="n">
+      <c r="H19" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I19" s="27" t="n"/>
-      <c r="J19" s="27" t="n">
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="K19" s="27" t="n">
+      <c r="K19" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="L19" s="27" t="n">
+      <c r="L19" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M19" s="27" t="n"/>
-      <c r="N19" s="27" t="n">
+      <c r="M19" s="32" t="n"/>
+      <c r="N19" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O19" s="27" t="n">
+      <c r="O19" s="32" t="n">
         <v>0.055</v>
       </c>
-      <c r="P19" s="27" t="n">
+      <c r="P19" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q19" s="27" t="n">
+      <c r="Q19" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="R19" s="27" t="n"/>
-      <c r="S19" s="27" t="n"/>
+      <c r="R19" s="32" t="n"/>
+      <c r="S19" s="32" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1739,57 +1754,57 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Carlos Toys</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="25" t="n">
+      <c r="C20" s="29" t="n"/>
+      <c r="D20" s="30" t="n">
         <v>4000000</v>
       </c>
-      <c r="E20" s="26" t="n">
+      <c r="E20" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="32" t="n">
         <v>0.49</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I20" s="27" t="n"/>
-      <c r="J20" s="27" t="n">
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="K20" s="27" t="n">
+      <c r="K20" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="L20" s="27" t="n">
+      <c r="L20" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M20" s="27" t="n"/>
-      <c r="N20" s="27" t="n">
+      <c r="M20" s="32" t="n"/>
+      <c r="N20" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O20" s="27" t="n">
+      <c r="O20" s="32" t="n">
         <v>0.055</v>
       </c>
-      <c r="P20" s="27" t="n">
+      <c r="P20" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q20" s="27" t="n">
+      <c r="Q20" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="R20" s="27" t="n"/>
-      <c r="S20" s="27" t="n"/>
+      <c r="R20" s="32" t="n"/>
+      <c r="S20" s="32" t="n"/>
       <c r="T20" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1797,57 +1812,57 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Kaloni</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="25" t="n">
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="30" t="n">
         <v>4000000</v>
       </c>
-      <c r="E21" s="26" t="n">
+      <c r="E21" s="31" t="n">
         <v>60000</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="32" t="n">
         <v>0.43</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="32" t="n">
         <v>0.49</v>
       </c>
-      <c r="H21" s="27" t="n">
+      <c r="H21" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="I21" s="27" t="n"/>
-      <c r="J21" s="27" t="n">
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="K21" s="27" t="n">
+      <c r="K21" s="32" t="n">
         <v>0.018</v>
       </c>
-      <c r="L21" s="27" t="n">
+      <c r="L21" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M21" s="27" t="n"/>
-      <c r="N21" s="27" t="n">
+      <c r="M21" s="32" t="n"/>
+      <c r="N21" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O21" s="27" t="n">
+      <c r="O21" s="32" t="n">
         <v>0.055</v>
       </c>
-      <c r="P21" s="27" t="n">
+      <c r="P21" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q21" s="27" t="n">
+      <c r="Q21" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="R21" s="27" t="n"/>
-      <c r="S21" s="27" t="n"/>
+      <c r="R21" s="32" t="n"/>
+      <c r="S21" s="32" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1855,63 +1870,63 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Bobois</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="25" t="n">
+      <c r="C22" s="29" t="n"/>
+      <c r="D22" s="30" t="n">
         <v>6000000</v>
       </c>
-      <c r="E22" s="26" t="n">
+      <c r="E22" s="31" t="n">
         <v>800</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="32" t="n">
         <v>0.48</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="I22" s="27" t="n">
+      <c r="I22" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="J22" s="27" t="n">
+      <c r="J22" s="32" t="n">
         <v>0.015</v>
       </c>
-      <c r="K22" s="27" t="n">
+      <c r="K22" s="32" t="n">
         <v>0.0185</v>
       </c>
-      <c r="L22" s="27" t="n">
+      <c r="L22" s="32" t="n">
         <v>0.029</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="N22" s="27" t="n">
+      <c r="N22" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="O22" s="27" t="n">
+      <c r="O22" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="P22" s="27" t="n">
+      <c r="P22" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q22" s="27" t="n">
+      <c r="Q22" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="R22" s="27" t="n">
+      <c r="R22" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S22" s="27" t="n"/>
+      <c r="S22" s="32" t="n"/>
       <c r="T22" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario 24 horas '. Competidor no nombrado ('Solución actual'). TPV = B2 (6M), ticket = B3. Shares TD B5, TC B6, AMEX B7, Internacional = Débito B8 + Crédito B9 (0.5% + 0.5%). MSI 0% (B10). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%) - ambos 3.0%. Sobretasas MSI K17:K22 (3x con Citi 5% y 3x 5%; 18x 18.9%). 24x no aparece. Otras hojas (Escenario 1, 48 horas, citi 3x, Hoja2) tienen valores distintos.</t>
@@ -1919,57 +1934,57 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>ARIAT</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="25" t="n">
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="30" t="n">
         <v>1800000</v>
       </c>
-      <c r="E23" s="26" t="n">
+      <c r="E23" s="31" t="n">
         <v>3800</v>
       </c>
-      <c r="F23" s="27" t="n">
+      <c r="F23" s="32" t="n">
         <v>0.19</v>
       </c>
-      <c r="G23" s="27" t="n">
+      <c r="G23" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="H23" s="27" t="n">
+      <c r="H23" s="32" t="n">
         <v>0.01</v>
       </c>
-      <c r="I23" s="27" t="n"/>
-      <c r="J23" s="27" t="n">
+      <c r="I23" s="32" t="n"/>
+      <c r="J23" s="32" t="n">
         <v>0.025</v>
       </c>
-      <c r="K23" s="27" t="n">
+      <c r="K23" s="32" t="n">
         <v>0.025</v>
       </c>
-      <c r="L23" s="27" t="n">
+      <c r="L23" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M23" s="27" t="n"/>
-      <c r="N23" s="27" t="n">
+      <c r="M23" s="32" t="n"/>
+      <c r="N23" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O23" s="27" t="n">
+      <c r="O23" s="32" t="n">
         <v>0.055</v>
       </c>
-      <c r="P23" s="27" t="n">
+      <c r="P23" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q23" s="27" t="n">
+      <c r="Q23" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="R23" s="27" t="n"/>
-      <c r="S23" s="27" t="n"/>
+      <c r="R23" s="32" t="n"/>
+      <c r="S23" s="32" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja '24h'. Competidor no nombrado ('Solución actual'). TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 1% B8 sin columna). Débito B17, Crédito B18, AMEX B19. Sobretasas MSI K17:K21. Sin Internacional, 18x ni 24x. Suma de shares = 101%. OP (TPV 400k) no incluido.</t>
@@ -1977,63 +1992,63 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="28" t="inlineStr">
         <is>
           <t>Petrolab</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="25" t="n">
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="30" t="n">
         <v>4000000</v>
       </c>
-      <c r="E24" s="26" t="n">
+      <c r="E24" s="31" t="n">
         <v>1500</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F24" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="G24" s="27" t="n">
+      <c r="G24" s="32" t="n">
         <v>0.27</v>
       </c>
-      <c r="H24" s="27" t="n">
+      <c r="H24" s="32" t="n">
         <v>0.13</v>
       </c>
-      <c r="I24" s="27" t="n">
+      <c r="I24" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="27" t="n">
+      <c r="J24" s="32" t="n">
         <v>0.0191</v>
       </c>
-      <c r="K24" s="27" t="n">
+      <c r="K24" s="32" t="n">
         <v>0.0218</v>
       </c>
-      <c r="L24" s="27" t="n">
+      <c r="L24" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M24" s="27" t="n">
+      <c r="M24" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="N24" s="27" t="n">
+      <c r="N24" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="O24" s="27" t="n">
+      <c r="O24" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="P24" s="27" t="n">
+      <c r="P24" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q24" s="27" t="n">
+      <c r="Q24" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="R24" s="27" t="n">
+      <c r="R24" s="32" t="n">
         <v>0.189</v>
       </c>
-      <c r="S24" s="27" t="n"/>
+      <c r="S24" s="32" t="n"/>
       <c r="T24" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Hoja1'. Competidor no nombrado ('Solución actual'). TPV = B2 ('Procesamiento'), ticket = B3. Shares TD B5, TC B6, AMEX B7, Int = Débito B8 + Crédito B9 (0%). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%). Sobretasas MSI J17:J22. 24x no aparece. OP (TPV 100k) no incluido.</t>
@@ -2041,63 +2056,63 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>Reina Diaz</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="25" t="n">
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="30" t="n">
         <v>800000</v>
       </c>
-      <c r="E25" s="26" t="n">
+      <c r="E25" s="31" t="n">
         <v>3800</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="32" t="n">
         <v>0.2</v>
       </c>
-      <c r="G25" s="27" t="n">
+      <c r="G25" s="32" t="n">
         <v>0.79</v>
       </c>
-      <c r="H25" s="27" t="n">
+      <c r="H25" s="32" t="n">
         <v>0.02</v>
       </c>
-      <c r="I25" s="27" t="n">
+      <c r="I25" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="27" t="n">
+      <c r="J25" s="32" t="n">
         <v>0.0169</v>
       </c>
-      <c r="K25" s="27" t="n">
+      <c r="K25" s="32" t="n">
         <v>0.0213</v>
       </c>
-      <c r="L25" s="27" t="n">
+      <c r="L25" s="32" t="n">
         <v>0.0285</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="N25" s="27" t="n">
+      <c r="N25" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="O25" s="27" t="n">
+      <c r="O25" s="32" t="n">
         <v>0.05</v>
       </c>
-      <c r="P25" s="27" t="n">
+      <c r="P25" s="32" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q25" s="27" t="n">
+      <c r="Q25" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="R25" s="27" t="n">
+      <c r="R25" s="32" t="n">
         <v>0.15</v>
       </c>
-      <c r="S25" s="27" t="n">
+      <c r="S25" s="32" t="n">
         <v>0.189</v>
       </c>
       <c r="T25" s="7" t="inlineStr">
@@ -2107,59 +2122,59 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>JULIO CEPEDA</t>
         </is>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="28" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="25" t="n">
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="30" t="n">
         <v>1000000</v>
       </c>
-      <c r="E26" s="26" t="n">
+      <c r="E26" s="31" t="n">
         <v>700</v>
       </c>
-      <c r="F26" s="27" t="n">
+      <c r="F26" s="32" t="n">
         <v>0.33</v>
       </c>
-      <c r="G26" s="27" t="n">
+      <c r="G26" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="H26" s="27" t="n">
+      <c r="H26" s="32" t="n">
         <v>0.1</v>
       </c>
-      <c r="I26" s="27" t="n"/>
-      <c r="J26" s="27" t="n">
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="32" t="n">
         <v>0.0137</v>
       </c>
-      <c r="K26" s="27" t="n">
+      <c r="K26" s="32" t="n">
         <v>0.019</v>
       </c>
-      <c r="L26" s="27" t="n">
+      <c r="L26" s="32" t="n">
         <v>0.03</v>
       </c>
-      <c r="M26" s="27" t="n"/>
-      <c r="N26" s="27" t="n">
+      <c r="M26" s="32" t="n"/>
+      <c r="N26" s="32" t="n">
         <v>0.032</v>
       </c>
-      <c r="O26" s="27" t="n">
+      <c r="O26" s="32" t="n">
         <v>0.0395</v>
       </c>
-      <c r="P26" s="27" t="n">
+      <c r="P26" s="32" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q26" s="27" t="n">
+      <c r="Q26" s="32" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="R26" s="27" t="n">
+      <c r="R26" s="32" t="n">
         <v>0.11</v>
       </c>
-      <c r="S26" s="27" t="n"/>
+      <c r="S26" s="32" t="n"/>
       <c r="T26" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Sin MSIs'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B6, TC B7, AMEX B8 (MSI 3% B9 sin columna). Débito B13, Crédito B14, AMEX B15. Sobretasas MSI K13:K17 (3x con Citi 3.2%, 3x 3.95%). Sin Internacional, 18x ni 24x. Suma de shares = 86%. Hoja 'MSIs' no revisada.</t>
@@ -2536,6 +2551,474 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="33" t="inlineStr">
+        <is>
+          <t>HI TEK</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C33" s="34" t="n"/>
+      <c r="D33" s="35" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E33" s="36" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F33" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G33" s="37" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H33" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I33" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="37" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="K33" s="37" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="L33" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M33" s="37" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N33" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O33" s="37" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="P33" s="37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q33" s="37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R33" s="37" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="S33" s="37" t="n"/>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int 0 (B8, B9), MSI 20% (B10) sin columna. Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (2.0%), Int Débito B21 (2.0%). Sobretasas MSI J17:J22. Sin 24x. OP no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t>DHI Clinic</t>
+        </is>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C34" s="34" t="n"/>
+      <c r="D34" s="35" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E34" s="36" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F34" s="37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G34" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I34" s="37" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J34" s="37" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="K34" s="37" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="L34" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M34" s="37" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="N34" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O34" s="37" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="P34" s="37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q34" s="37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R34" s="37" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="S34" s="37" t="n"/>
+      <c r="T34" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6 (0%), AMEX B7, Int = Débito B8 (30%) + Crédito B9 (57%) = 87%. Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (2.5%), Int Débito B21 (2.5%). Sobretasas MSI J17:J22. Sin 24x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>Diagsa</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C35" s="34" t="n"/>
+      <c r="D35" s="35" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E35" s="36" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F35" s="37" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G35" s="37" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="H35" s="37" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="I35" s="37" t="n"/>
+      <c r="J35" s="37" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="K35" s="37" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="L35" s="37" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M35" s="37" t="n"/>
+      <c r="N35" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O35" s="37" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P35" s="37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Q35" s="37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R35" s="37" t="n"/>
+      <c r="S35" s="37" t="n"/>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>Origen: Hoja1. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 2% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J15 (meses en numérico 3/6/9/12). Sin Internacional, 18x ni 24x. OP no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="33" t="inlineStr">
+        <is>
+          <t>Christus</t>
+        </is>
+      </c>
+      <c r="B36" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="35" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F36" s="37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G36" s="37" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H36" s="37" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I36" s="37" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J36" s="37" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="K36" s="37" t="n">
+        <v>0.0158</v>
+      </c>
+      <c r="L36" s="37" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="M36" s="37" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="N36" s="37" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="O36" s="37" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="P36" s="37" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="Q36" s="37" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="R36" s="37" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S36" s="37" t="n"/>
+      <c r="T36" s="7" t="inlineStr">
+        <is>
+          <t>Origen: hoja 'Monetizacion OP+ Débito', bloque terminales. TPV = B2 (45M total; B3 Débito+MSI 15.75M y B4 Procesamiento 12.25M, confirmar). Ticket B5 = 50,000 (revisar). Shares TD B7, TC B8, AMEX B9, Int Débito B10 (MSI 5% B14 y MP 1% B11 sin columna; suma &gt;100%). Débito B24, Crédito B25, AMEX B26, Int B27. Sobretasas MSI K24:K29. 24x no aparece. Bloque OP no incluido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="33" t="inlineStr">
+        <is>
+          <t>Colibrí BEBE</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C37" s="34" t="inlineStr">
+        <is>
+          <t>Apparel</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="n"/>
+      <c r="E37" s="36" t="n"/>
+      <c r="F37" s="37" t="n"/>
+      <c r="G37" s="37" t="n"/>
+      <c r="H37" s="37" t="n"/>
+      <c r="I37" s="37" t="n"/>
+      <c r="J37" s="37" t="n">
+        <v>0.0174</v>
+      </c>
+      <c r="K37" s="37" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="L37" s="37" t="n"/>
+      <c r="M37" s="37" t="n"/>
+      <c r="N37" s="37" t="n"/>
+      <c r="O37" s="37" t="n"/>
+      <c r="P37" s="37" t="n"/>
+      <c r="Q37" s="37" t="n"/>
+      <c r="R37" s="37" t="n"/>
+      <c r="S37" s="37" t="n"/>
+      <c r="T37" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto (hoja compartida). Débito 1.74%, Crédito 2.30%, AMEX vacío. Sin TPV, shares ni MSI en la foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="33" t="inlineStr">
+        <is>
+          <t>Alessia</t>
+        </is>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C38" s="34" t="inlineStr">
+        <is>
+          <t>Automotriz y refacciones</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="n"/>
+      <c r="E38" s="36" t="n"/>
+      <c r="F38" s="37" t="n"/>
+      <c r="G38" s="37" t="n"/>
+      <c r="H38" s="37" t="n"/>
+      <c r="I38" s="37" t="n"/>
+      <c r="J38" s="37" t="n">
+        <v>0.0181</v>
+      </c>
+      <c r="K38" s="37" t="n">
+        <v>0.0258</v>
+      </c>
+      <c r="L38" s="37" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="M38" s="37" t="n"/>
+      <c r="N38" s="37" t="n"/>
+      <c r="O38" s="37" t="n"/>
+      <c r="P38" s="37" t="n"/>
+      <c r="Q38" s="37" t="n"/>
+      <c r="R38" s="37" t="n"/>
+      <c r="S38" s="37" t="n"/>
+      <c r="T38" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto. Crédito muestra 2.58% y debajo 3.51% en la misma celda; guardé 2.58% y el 3.51% no se identifica (¿otro crédito o MSI?). AMEX 3.51%. Industria cortada en la foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="33" t="inlineStr">
+        <is>
+          <t>Jump In</t>
+        </is>
+      </c>
+      <c r="B39" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C39" s="34" t="inlineStr">
+        <is>
+          <t>Entretenimiento</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="n"/>
+      <c r="E39" s="36" t="n"/>
+      <c r="F39" s="37" t="n"/>
+      <c r="G39" s="37" t="n"/>
+      <c r="H39" s="37" t="n"/>
+      <c r="I39" s="37" t="n"/>
+      <c r="J39" s="37" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K39" s="37" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L39" s="37" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="M39" s="37" t="n"/>
+      <c r="N39" s="37" t="n"/>
+      <c r="O39" s="37" t="n"/>
+      <c r="P39" s="37" t="n"/>
+      <c r="Q39" s="37" t="n"/>
+      <c r="R39" s="37" t="n"/>
+      <c r="S39" s="37" t="n"/>
+      <c r="T39" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto. Débito se ve como '0,02' sin % (guardé 2%, confirmar si es 0.02% o 2%). Crédito 2%, AMEX 2.6%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="33" t="inlineStr">
+        <is>
+          <t>Rodango</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C40" s="34" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="37" t="n"/>
+      <c r="G40" s="37" t="n"/>
+      <c r="H40" s="37" t="n"/>
+      <c r="I40" s="37" t="n"/>
+      <c r="J40" s="37" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="K40" s="37" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="L40" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M40" s="37" t="n"/>
+      <c r="N40" s="37" t="n"/>
+      <c r="O40" s="37" t="n"/>
+      <c r="P40" s="37" t="n"/>
+      <c r="Q40" s="37" t="n"/>
+      <c r="R40" s="37" t="n"/>
+      <c r="S40" s="37" t="n"/>
+      <c r="T40" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto. Débito 1.5%, Crédito 1.7%, AMEX 3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="33" t="inlineStr">
+        <is>
+          <t>DNI Interiores</t>
+        </is>
+      </c>
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C41" s="34" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D41" s="35" t="n"/>
+      <c r="E41" s="36" t="n"/>
+      <c r="F41" s="37" t="n"/>
+      <c r="G41" s="37" t="n"/>
+      <c r="H41" s="37" t="n"/>
+      <c r="I41" s="37" t="n"/>
+      <c r="J41" s="37" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="K41" s="37" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="L41" s="37" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M41" s="37" t="n"/>
+      <c r="N41" s="37" t="n"/>
+      <c r="O41" s="37" t="n"/>
+      <c r="P41" s="37" t="n"/>
+      <c r="Q41" s="37" t="n"/>
+      <c r="R41" s="37" t="n"/>
+      <c r="S41" s="37" t="n"/>
+      <c r="T41" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto. Débito 1.5%, Crédito 1.7%, AMEX 3%.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Svenson and Muebleria Corra rows from photo (Publico omitted)
Claude-Session: https://claude.ai/code/session_01M2tL3DwZ7DqXaetV3JS43c
</commit_message>
<xml_diff>
--- a/output/tasas_competidores.xlsx
+++ b/output/tasas_competidores.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -554,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T41"/>
+  <dimension ref="A1:T43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -682,55 +697,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>VANS (NO VIGENTE)</t>
         </is>
       </c>
-      <c r="B2" s="28" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C2" s="29" t="n"/>
-      <c r="D2" s="30" t="n">
+      <c r="C2" s="34" t="n"/>
+      <c r="D2" s="35" t="n">
         <v>77945500</v>
       </c>
-      <c r="E2" s="31" t="n"/>
-      <c r="F2" s="32" t="n">
+      <c r="E2" s="36" t="n"/>
+      <c r="F2" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G2" s="32" t="n">
+      <c r="G2" s="37" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="32" t="n">
+      <c r="H2" s="37" t="n">
         <v>0.02</v>
       </c>
-      <c r="I2" s="32" t="n">
+      <c r="I2" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="32" t="n">
+      <c r="J2" s="37" t="n">
         <v>0.015</v>
       </c>
-      <c r="K2" s="32" t="n"/>
-      <c r="L2" s="32" t="n"/>
-      <c r="M2" s="32" t="n"/>
-      <c r="N2" s="32" t="n">
+      <c r="K2" s="37" t="n"/>
+      <c r="L2" s="37" t="n"/>
+      <c r="M2" s="37" t="n"/>
+      <c r="N2" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O2" s="32" t="n">
+      <c r="O2" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P2" s="32" t="n">
+      <c r="P2" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q2" s="32" t="n">
+      <c r="Q2" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R2" s="32" t="n">
+      <c r="R2" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S2" s="32" t="n"/>
+      <c r="S2" s="37" t="n"/>
       <c r="T2" s="7" t="inlineStr">
         <is>
           <t>NO VIGENTE (reemplazada por VANS - 1). Origen: 'Monetización'. TPV = B3 ('Grupo', confirmar). Débito = B25. MSI = sobretasas L36:L40. Base TC (B36) vacía. 24x no aparece.</t>
@@ -738,61 +753,61 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="33" t="inlineStr">
         <is>
           <t>VANS - 1 (VIGENTE)</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C3" s="29" t="n"/>
-      <c r="D3" s="30" t="n">
+      <c r="C3" s="34" t="n"/>
+      <c r="D3" s="35" t="n">
         <v>77945500</v>
       </c>
-      <c r="E3" s="31" t="n"/>
-      <c r="F3" s="32" t="n">
+      <c r="E3" s="36" t="n"/>
+      <c r="F3" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G3" s="32" t="n">
+      <c r="G3" s="37" t="n">
         <v>0.51</v>
       </c>
-      <c r="H3" s="32" t="n">
+      <c r="H3" s="37" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" s="32" t="n">
+      <c r="I3" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="32" t="n">
+      <c r="J3" s="37" t="n">
         <v>0.0142</v>
       </c>
-      <c r="K3" s="32" t="n">
+      <c r="K3" s="37" t="n">
         <v>0.0202</v>
       </c>
-      <c r="L3" s="32" t="n">
+      <c r="L3" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M3" s="32" t="n">
+      <c r="M3" s="37" t="n">
         <v>0.0202</v>
       </c>
-      <c r="N3" s="32" t="n">
+      <c r="N3" s="37" t="n">
         <v>0.0493</v>
       </c>
-      <c r="O3" s="32" t="n">
+      <c r="O3" s="37" t="n">
         <v>0.0842</v>
       </c>
-      <c r="P3" s="32" t="n">
+      <c r="P3" s="37" t="n">
         <v>0.1174</v>
       </c>
-      <c r="Q3" s="32" t="n">
+      <c r="Q3" s="37" t="n">
         <v>0.1491</v>
       </c>
-      <c r="R3" s="32" t="n">
+      <c r="R3" s="37" t="n">
         <v>0.19</v>
       </c>
-      <c r="S3" s="32" t="n"/>
+      <c r="S3" s="37" t="n"/>
       <c r="T3" s="7" t="inlineStr">
         <is>
           <t>VIGENTE. Origen: MONETIZAR_-_VANS_-_1, 'Escenario 1'. TPV = B2 ('Grupo'). Débito B20, Crédito B21, AMEX B22, Internacional B23. Sobretasas MSI L21:L25. 24x no aparece. Ticket vacío.</t>
@@ -800,61 +815,61 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C4" s="29" t="n"/>
-      <c r="D4" s="30" t="n">
+      <c r="C4" s="34" t="n"/>
+      <c r="D4" s="35" t="n">
         <v>9213568.4673</v>
       </c>
-      <c r="E4" s="31" t="n">
+      <c r="E4" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="37" t="n">
         <v>0.2758</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="37" t="n">
         <v>0.1315</v>
       </c>
-      <c r="H4" s="32" t="n"/>
-      <c r="I4" s="32" t="n">
+      <c r="H4" s="37" t="n"/>
+      <c r="I4" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="32" t="n">
+      <c r="J4" s="37" t="n">
         <v>0.014</v>
       </c>
-      <c r="K4" s="32" t="n">
+      <c r="K4" s="37" t="n">
         <v>0.017</v>
       </c>
-      <c r="L4" s="32" t="n">
+      <c r="L4" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M4" s="32" t="n">
+      <c r="M4" s="37" t="n">
         <v>0.034</v>
       </c>
-      <c r="N4" s="32" t="n">
+      <c r="N4" s="37" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O4" s="32" t="n">
+      <c r="O4" s="37" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P4" s="32" t="n">
+      <c r="P4" s="37" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q4" s="32" t="n">
+      <c r="Q4" s="37" t="n">
         <v>0.12</v>
       </c>
-      <c r="R4" s="32" t="n">
+      <c r="R4" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S4" s="32" t="n"/>
+      <c r="S4" s="37" t="n"/>
       <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%'. TPV = B2 x C3 (BBVA = TD+TC+MSI). Share TD B7, TC B8. Débito B25, Crédito B26, AMEX B27, Internacional B28. Sobretasas MSI K25:K30 (3x usa '3x' K26; 3x con Citi K25 también 5.01%). BBVA MSI 2.16% (B9) sin columna. 24x no aparece. Hojas '0.55%' y 'Ejercicio' tienen variantes de MP.</t>
@@ -862,59 +877,59 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>San Angel INN 2 terminales</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>MIFEL</t>
         </is>
       </c>
-      <c r="C5" s="29" t="n"/>
-      <c r="D5" s="30" t="n">
+      <c r="C5" s="34" t="n"/>
+      <c r="D5" s="35" t="n">
         <v>11838651.3927</v>
       </c>
-      <c r="E5" s="31" t="n">
+      <c r="E5" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="37" t="n">
         <v>0.3652</v>
       </c>
-      <c r="G5" s="32" t="n">
+      <c r="G5" s="37" t="n">
         <v>0.164</v>
       </c>
-      <c r="H5" s="32" t="n">
+      <c r="H5" s="37" t="n">
         <v>0.008</v>
       </c>
-      <c r="I5" s="32" t="n">
+      <c r="I5" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="32" t="n">
+      <c r="J5" s="37" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K5" s="32" t="n">
+      <c r="K5" s="37" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L5" s="32" t="n"/>
-      <c r="M5" s="32" t="n"/>
-      <c r="N5" s="32" t="n">
+      <c r="L5" s="37" t="n"/>
+      <c r="M5" s="37" t="n"/>
+      <c r="N5" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O5" s="32" t="n">
+      <c r="O5" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P5" s="32" t="n">
+      <c r="P5" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q5" s="32" t="n">
+      <c r="Q5" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R5" s="32" t="n">
+      <c r="R5" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S5" s="32" t="n"/>
+      <c r="S5" s="37" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion 0.50%', sección MIFEL. TPV = B2 x C4 (DEBMIFEL+CREMIFEL+AMEX+MSI mifel). Share TD = DEBMIFEL B10, TC = CREMIFEL B11, AMEX B12. Débito B38, Crédito B39. Sobretasas MSI K38:K43. Sin tasa AMEX/Internacional. MSI mifel 1.39% (B13) sin columna. 24x no aparece.</t>
@@ -922,53 +937,53 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="33" t="inlineStr">
         <is>
           <t>Santander</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="30" t="n">
+      <c r="C6" s="34" t="n"/>
+      <c r="D6" s="35" t="n">
         <v>36864986.512</v>
       </c>
-      <c r="E6" s="31" t="n">
+      <c r="E6" s="36" t="n">
         <v>544</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F6" s="37" t="n">
         <v>0.6686303192319475</v>
       </c>
-      <c r="G6" s="32" t="n"/>
-      <c r="H6" s="32" t="n">
+      <c r="G6" s="37" t="n"/>
+      <c r="H6" s="37" t="n">
         <v>0.01490860168417793</v>
       </c>
-      <c r="I6" s="32" t="n">
+      <c r="I6" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="32" t="n">
+      <c r="J6" s="37" t="n">
         <v>0.016</v>
       </c>
-      <c r="K6" s="32" t="n">
+      <c r="K6" s="37" t="n">
         <v>0.02</v>
       </c>
-      <c r="L6" s="32" t="n">
+      <c r="L6" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="M6" s="32" t="n"/>
-      <c r="N6" s="32" t="n">
+      <c r="M6" s="37" t="n"/>
+      <c r="N6" s="37" t="n">
         <v>0.033</v>
       </c>
-      <c r="O6" s="32" t="n">
+      <c r="O6" s="37" t="n">
         <v>0.048</v>
       </c>
-      <c r="P6" s="32" t="n"/>
-      <c r="Q6" s="32" t="n"/>
-      <c r="R6" s="32" t="n"/>
-      <c r="S6" s="32" t="n"/>
+      <c r="P6" s="37" t="n"/>
+      <c r="Q6" s="37" t="n"/>
+      <c r="R6" s="37" t="n"/>
+      <c r="S6" s="37" t="n"/>
       <c r="T6" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia'. TPV = B2 x C3 (95%). Share TD = C7 ($25,946,366) / B2 calculado; AMEX = C12 ($578,532) / B2 calculado. TC Santander no aparece. Débito B25, Crédito B26, AMEX B27. Sobretasas MSI H26:K27 (solo 3x y 6x). Internacional sin tasa. Hoja '24 horas' tiene variantes de tasas.</t>
@@ -976,45 +991,45 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>VEANNA</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="30" t="n">
+      <c r="C7" s="34" t="n"/>
+      <c r="D7" s="35" t="n">
         <v>1940262.448</v>
       </c>
-      <c r="E7" s="31" t="n">
+      <c r="E7" s="36" t="n">
         <v>544</v>
       </c>
-      <c r="F7" s="32" t="n"/>
-      <c r="G7" s="32" t="n"/>
-      <c r="H7" s="32" t="n"/>
-      <c r="I7" s="32" t="n"/>
-      <c r="J7" s="32" t="n">
+      <c r="F7" s="37" t="n"/>
+      <c r="G7" s="37" t="n"/>
+      <c r="H7" s="37" t="n"/>
+      <c r="I7" s="37" t="n"/>
+      <c r="J7" s="37" t="n">
         <v>0.0136</v>
       </c>
-      <c r="K7" s="32" t="n">
+      <c r="K7" s="37" t="n">
         <v>0.0181</v>
       </c>
-      <c r="L7" s="32" t="n"/>
-      <c r="M7" s="32" t="n"/>
-      <c r="N7" s="32" t="n">
+      <c r="L7" s="37" t="n"/>
+      <c r="M7" s="37" t="n"/>
+      <c r="N7" s="37" t="n">
         <v>0.0355</v>
       </c>
-      <c r="O7" s="32" t="n">
+      <c r="O7" s="37" t="n">
         <v>0.0735</v>
       </c>
-      <c r="P7" s="32" t="n"/>
-      <c r="Q7" s="32" t="n"/>
-      <c r="R7" s="32" t="n"/>
-      <c r="S7" s="32" t="n"/>
+      <c r="P7" s="37" t="n"/>
+      <c r="Q7" s="37" t="n"/>
+      <c r="R7" s="37" t="n"/>
+      <c r="S7" s="37" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Ejercicio  Monetizacion Inmedia', sección BBVA. TPV = B2 x C4 (5%, 'BBVA MSI'). Débito B38, Crédito B39. Sobretasas MSI K39:K40 (solo 3x y 6x). Shares de BBVA no vienen en el archivo.</t>
@@ -1022,57 +1037,57 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Aguillon</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>CLIP</t>
         </is>
       </c>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="30" t="n">
+      <c r="C8" s="34" t="n"/>
+      <c r="D8" s="35" t="n">
         <v>300000</v>
       </c>
-      <c r="E8" s="31" t="n">
+      <c r="E8" s="36" t="n">
         <v>3500</v>
       </c>
-      <c r="F8" s="32" t="n">
+      <c r="F8" s="37" t="n">
         <v>0.45</v>
       </c>
-      <c r="G8" s="32" t="n">
+      <c r="G8" s="37" t="n">
         <v>0.3</v>
       </c>
-      <c r="H8" s="32" t="n"/>
-      <c r="I8" s="32" t="n"/>
-      <c r="J8" s="32" t="n">
+      <c r="H8" s="37" t="n"/>
+      <c r="I8" s="37" t="n"/>
+      <c r="J8" s="37" t="n">
         <v>0.028</v>
       </c>
-      <c r="K8" s="32" t="n">
+      <c r="K8" s="37" t="n">
         <v>0.028</v>
       </c>
-      <c r="L8" s="32" t="n">
+      <c r="L8" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M8" s="32" t="n">
+      <c r="M8" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="N8" s="32" t="n">
+      <c r="N8" s="37" t="n">
         <v>0.0457</v>
       </c>
-      <c r="O8" s="32" t="n">
+      <c r="O8" s="37" t="n">
         <v>0.0757</v>
       </c>
-      <c r="P8" s="32" t="n">
+      <c r="P8" s="37" t="n">
         <v>0.1107</v>
       </c>
-      <c r="Q8" s="32" t="n">
+      <c r="Q8" s="37" t="n">
         <v>0.1277</v>
       </c>
-      <c r="R8" s="32" t="n"/>
-      <c r="S8" s="32" t="n"/>
+      <c r="R8" s="37" t="n"/>
+      <c r="S8" s="37" t="n"/>
       <c r="T8" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion Clip'. TPV = B2 'Total' (300,000); B3 'Procesamiento' = 500,000, . Share TD B6, TC B7 (MSI 25% sin columna). Débito B17, Crédito B18, AMEX B19 (sin etiqueta, asumido AMEX), Internacional B20. Sobretasas MSI K17:K20. 18x sin sobretasa en el archivo. Filas 74-122 ocultas, sin datos. TPV mensual (confirmado por el usuario).</t>
@@ -1080,61 +1095,61 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="30" t="n">
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="35" t="n">
         <v>40000000</v>
       </c>
-      <c r="E9" s="31" t="n"/>
-      <c r="F9" s="32" t="n">
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="37" t="n">
         <v>0.29</v>
       </c>
-      <c r="G9" s="32" t="n">
+      <c r="G9" s="37" t="n">
         <v>0.35</v>
       </c>
-      <c r="H9" s="32" t="n">
+      <c r="H9" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I9" s="32" t="n">
+      <c r="I9" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J9" s="32" t="n">
+      <c r="J9" s="37" t="n">
         <v>0.0115</v>
       </c>
-      <c r="K9" s="32" t="n">
+      <c r="K9" s="37" t="n">
         <v>0.0167</v>
       </c>
-      <c r="L9" s="32" t="n">
+      <c r="L9" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="M9" s="32" t="n">
+      <c r="M9" s="37" t="n">
         <v>0.025</v>
       </c>
-      <c r="N9" s="32" t="n">
+      <c r="N9" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O9" s="32" t="n">
+      <c r="O9" s="37" t="n">
         <v>0.048</v>
       </c>
-      <c r="P9" s="32" t="n">
+      <c r="P9" s="37" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q9" s="32" t="n">
+      <c r="Q9" s="37" t="n">
         <v>0.105</v>
       </c>
-      <c r="R9" s="32" t="n">
+      <c r="R9" s="37" t="n">
         <v>0.16</v>
       </c>
-      <c r="S9" s="32" t="n"/>
+      <c r="S9" s="37" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección BBVA. TPV = B3 'Grupo' (mensual, confirmado por el usuario). Share TD B7, TC B8, AMEX B9, Int B12 (MSI 26% y MP 1% sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. Ticket vacío. 24x no aparece. Hoja 'Dif Tasas' es comparativa.</t>
@@ -1142,57 +1157,57 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>Auna</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="33" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C10" s="29" t="n"/>
-      <c r="D10" s="30" t="n">
+      <c r="C10" s="34" t="n"/>
+      <c r="D10" s="35" t="n">
         <v>40000000</v>
       </c>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="32" t="n">
+      <c r="E10" s="36" t="n"/>
+      <c r="F10" s="37" t="n">
         <v>0.29</v>
       </c>
-      <c r="G10" s="32" t="n">
+      <c r="G10" s="37" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" s="32" t="n">
+      <c r="H10" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I10" s="32" t="n">
+      <c r="I10" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J10" s="32" t="n">
+      <c r="J10" s="37" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K10" s="32" t="n">
+      <c r="K10" s="37" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="32" t="n"/>
-      <c r="N10" s="32" t="n">
+      <c r="L10" s="37" t="n"/>
+      <c r="M10" s="37" t="n"/>
+      <c r="N10" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O10" s="32" t="n">
+      <c r="O10" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P10" s="32" t="n">
+      <c r="P10" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q10" s="32" t="n">
+      <c r="Q10" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R10" s="32" t="n">
+      <c r="R10" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S10" s="32" t="n"/>
+      <c r="S10" s="37" t="n"/>
       <c r="T10" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Escenario 1', sección Fiserv. Mismo TPV y shares que BBVA (B3, B7:B12). Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin tasa AMEX/Internacional. 24x no aparece. TPV mensual (confirmado por el usuario).</t>
@@ -1200,63 +1215,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n"/>
-      <c r="D11" s="30" t="n">
+      <c r="C11" s="34" t="n"/>
+      <c r="D11" s="35" t="n">
         <v>136100110.57</v>
       </c>
-      <c r="E11" s="31" t="n">
+      <c r="E11" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F11" s="32" t="n">
+      <c r="F11" s="37" t="n">
         <v>0.6713</v>
       </c>
-      <c r="G11" s="32" t="n">
+      <c r="G11" s="37" t="n">
         <v>0.3075</v>
       </c>
-      <c r="H11" s="32" t="n">
+      <c r="H11" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="32" t="n">
+      <c r="I11" s="37" t="n">
         <v>0.0212</v>
       </c>
-      <c r="J11" s="32" t="n">
+      <c r="J11" s="37" t="n">
         <v>0.0145</v>
       </c>
-      <c r="K11" s="32" t="n">
+      <c r="K11" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="L11" s="32" t="n">
+      <c r="L11" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="M11" s="32" t="n">
+      <c r="M11" s="37" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N11" s="32" t="n">
+      <c r="N11" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O11" s="32" t="n">
+      <c r="O11" s="37" t="n">
         <v>0.075</v>
       </c>
-      <c r="P11" s="32" t="n">
+      <c r="P11" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q11" s="32" t="n">
+      <c r="Q11" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="R11" s="32" t="n">
+      <c r="R11" s="37" t="n">
         <v>0.18</v>
       </c>
-      <c r="S11" s="32" t="n"/>
+      <c r="S11" s="37" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%' (mensual, confirmado por el usuario). TPV mensual, confirmado por el usuario. Share TD B7, TC B8, Int BBVA B15. Débito B26, Crédito B27, AMEX B28, Int B29. Sobretasas MSI L26:L31 (3x con Citi = 3.5%). 24x no aparece.</t>
@@ -1264,61 +1279,61 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>HangTen 2</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C12" s="29" t="n"/>
-      <c r="D12" s="30" t="n">
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="35" t="n">
         <v>94010839.39</v>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E12" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F12" s="32" t="n">
+      <c r="F12" s="37" t="n">
         <v>0.6605</v>
       </c>
-      <c r="G12" s="32" t="n">
+      <c r="G12" s="37" t="n">
         <v>0.3389</v>
       </c>
-      <c r="H12" s="32" t="n">
+      <c r="H12" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="32" t="n">
+      <c r="I12" s="37" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="J12" s="32" t="n">
+      <c r="J12" s="37" t="n">
         <v>0.0144</v>
       </c>
-      <c r="K12" s="32" t="n">
+      <c r="K12" s="37" t="n">
         <v>0.0179</v>
       </c>
-      <c r="L12" s="32" t="n"/>
-      <c r="M12" s="32" t="n">
+      <c r="L12" s="37" t="n"/>
+      <c r="M12" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" s="32" t="n">
+      <c r="N12" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O12" s="32" t="n">
+      <c r="O12" s="37" t="n">
         <v>0.045</v>
       </c>
-      <c r="P12" s="32" t="n">
+      <c r="P12" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q12" s="32" t="n">
+      <c r="Q12" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R12" s="32" t="n">
+      <c r="R12" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S12" s="32" t="n"/>
+      <c r="S12" s="37" t="n"/>
       <c r="T12" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.45%', sección Fiserv (ANUAL). TPV mensual, confirmado por el usuario. Share DEB Fiserv B10, CRE B11, Int Fiserv B14. Débito B39, Crédito B40, Int B41. Sobretasas MSI L39:L44. 6x = 4.5% (fila 'Fiserv' 6x). Fila 'Fiserv' 6x con Citibanamex = 8.76% (L39), no mapeada. 24x no aparece.</t>
@@ -1326,63 +1341,63 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>Caso 3 soluciones</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="30" t="n">
+      <c r="C13" s="34" t="n"/>
+      <c r="D13" s="35" t="n">
         <v>10000000</v>
       </c>
-      <c r="E13" s="31" t="n">
+      <c r="E13" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F13" s="32" t="n">
+      <c r="F13" s="37" t="n">
         <v>0.5</v>
       </c>
-      <c r="G13" s="32" t="n">
+      <c r="G13" s="37" t="n">
         <v>0.28</v>
       </c>
-      <c r="H13" s="32" t="n">
+      <c r="H13" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="I13" s="32" t="n">
+      <c r="I13" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J13" s="32" t="n">
+      <c r="J13" s="37" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K13" s="32" t="n">
+      <c r="K13" s="37" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L13" s="32" t="n">
+      <c r="L13" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M13" s="32" t="n">
+      <c r="M13" s="37" t="n">
         <v>0.034</v>
       </c>
-      <c r="N13" s="32" t="n">
+      <c r="N13" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O13" s="32" t="n">
+      <c r="O13" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P13" s="32" t="n">
+      <c r="P13" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="32" t="n">
+      <c r="Q13" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R13" s="32" t="n">
+      <c r="R13" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S13" s="32" t="n"/>
+      <c r="S13" s="37" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
           <t>Origen: 'Monetizacion 0.55%', sección Fiserv. TPV = B2 (10M). Shares B10:B14 (Opción bancaria, iguales en Opción 1/2/3). Débito B49, Crédito B50, AMEX B51, Int B52. Sobretasas MSI K50:K54. 24x no aparece. Opción 1 = BBVA igual a San Angel; Opción 2 y 3 sin tasas en el archivo.</t>
@@ -1390,63 +1405,63 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="30" t="n">
+      <c r="C14" s="34" t="n"/>
+      <c r="D14" s="35" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E14" s="31" t="n">
+      <c r="E14" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F14" s="32" t="n">
+      <c r="F14" s="37" t="n">
         <v>0.75</v>
       </c>
-      <c r="G14" s="32" t="n">
+      <c r="G14" s="37" t="n">
         <v>0.24</v>
       </c>
-      <c r="H14" s="32" t="n">
+      <c r="H14" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="32" t="n">
+      <c r="I14" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J14" s="32" t="n">
+      <c r="J14" s="37" t="n">
         <v>0.0125</v>
       </c>
-      <c r="K14" s="32" t="n">
+      <c r="K14" s="37" t="n">
         <v>0.0161</v>
       </c>
-      <c r="L14" s="32" t="n">
+      <c r="L14" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="M14" s="32" t="n">
+      <c r="M14" s="37" t="n">
         <v>0.033</v>
       </c>
-      <c r="N14" s="32" t="n">
+      <c r="N14" s="37" t="n">
         <v>0.0501</v>
       </c>
-      <c r="O14" s="32" t="n">
+      <c r="O14" s="37" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P14" s="32" t="n">
+      <c r="P14" s="37" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q14" s="32" t="n">
+      <c r="Q14" s="37" t="n">
         <v>0.12</v>
       </c>
-      <c r="R14" s="32" t="n">
+      <c r="R14" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S14" s="32" t="n"/>
+      <c r="S14" s="37" t="n"/>
       <c r="T14" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo'. Merchant = CITI. TPV = B3 = B2/12 x C2 (B2 anual 295,435,191 / 12 x 100%). Shares TD B7, TC B8, Int B14. Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI L26:L30. 24x no aparece. Otras hojas: 'EscenarioPsycho' tiene TPV 32M y AMEX/Int distintos (2.6%/2.4%) y 3x 1.91%; 'Flujo Comp (2)' y '1.77-1.99' tienen tasas distintas.</t>
@@ -1454,59 +1469,59 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="33" t="inlineStr">
         <is>
           <t>Fiserv</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
-      <c r="D15" s="30" t="n">
+      <c r="C15" s="34" t="n"/>
+      <c r="D15" s="35" t="n">
         <v>24619599.25</v>
       </c>
-      <c r="E15" s="31" t="n">
+      <c r="E15" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F15" s="32" t="n">
+      <c r="F15" s="37" t="n">
         <v>0.75</v>
       </c>
-      <c r="G15" s="32" t="n">
+      <c r="G15" s="37" t="n">
         <v>0.24</v>
       </c>
-      <c r="H15" s="32" t="n">
+      <c r="H15" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="32" t="n">
+      <c r="I15" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J15" s="32" t="n">
+      <c r="J15" s="37" t="n">
         <v>0.0135</v>
       </c>
-      <c r="K15" s="32" t="n">
+      <c r="K15" s="37" t="n">
         <v>0.0165</v>
       </c>
-      <c r="L15" s="32" t="n"/>
-      <c r="M15" s="32" t="n"/>
-      <c r="N15" s="32" t="n">
+      <c r="L15" s="37" t="n"/>
+      <c r="M15" s="37" t="n"/>
+      <c r="N15" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O15" s="32" t="n">
+      <c r="O15" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P15" s="32" t="n">
+      <c r="P15" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q15" s="32" t="n">
+      <c r="Q15" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R15" s="32" t="n">
+      <c r="R15" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S15" s="32" t="n"/>
+      <c r="S15" s="37" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario Lineas Flujo Complejo', sección Fiserv. Mismo TPV y shares que BBVA. Débito B38, Crédito B39. Sobretasas MSI L38:L43 (3x con Citi = 3.5%). Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1514,63 +1529,63 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="30" t="n">
+      <c r="C16" s="34" t="n"/>
+      <c r="D16" s="35" t="n">
         <v>5200000</v>
       </c>
-      <c r="E16" s="31" t="n">
+      <c r="E16" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F16" s="32" t="n">
+      <c r="F16" s="37" t="n">
         <v>0.2</v>
       </c>
-      <c r="G16" s="32" t="n">
+      <c r="G16" s="37" t="n">
         <v>0.25</v>
       </c>
-      <c r="H16" s="32" t="n">
+      <c r="H16" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="32" t="n">
+      <c r="I16" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="32" t="n">
+      <c r="J16" s="37" t="n">
         <v>0.0175</v>
       </c>
-      <c r="K16" s="32" t="n">
+      <c r="K16" s="37" t="n">
         <v>0.0238</v>
       </c>
-      <c r="L16" s="32" t="n">
+      <c r="L16" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="M16" s="32" t="n">
+      <c r="M16" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="N16" s="32" t="n">
+      <c r="N16" s="37" t="n">
         <v>0.0553</v>
       </c>
-      <c r="O16" s="32" t="n">
+      <c r="O16" s="37" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="P16" s="32" t="n">
+      <c r="P16" s="37" t="n">
         <v>0.09</v>
       </c>
-      <c r="Q16" s="32" t="n">
+      <c r="Q16" s="37" t="n">
         <v>0.12</v>
       </c>
-      <c r="R16" s="32" t="n">
+      <c r="R16" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S16" s="32" t="n"/>
+      <c r="S16" s="37" t="n"/>
       <c r="T16" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ' (con espacio). TPV = B2 (8M) x C3 (65%). Share TD B7, TC B8 (BBVA MSI 10%, B9, sin columna). Débito B25, Crédito B26, AMEX B27, Int B28. Sobretasas MSI K26:K30. 24x no aparece. Sin periodo en el archivo (confirmar).</t>
@@ -1578,59 +1593,59 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>Vertex</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="33" t="inlineStr">
         <is>
           <t>Banamex</t>
         </is>
       </c>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="30" t="n">
+      <c r="C17" s="34" t="n"/>
+      <c r="D17" s="35" t="n">
         <v>2800000</v>
       </c>
-      <c r="E17" s="31" t="n">
+      <c r="E17" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F17" s="32" t="n">
+      <c r="F17" s="37" t="n">
         <v>0.2</v>
       </c>
-      <c r="G17" s="32" t="n">
+      <c r="G17" s="37" t="n">
         <v>0.25</v>
       </c>
-      <c r="H17" s="32" t="n">
+      <c r="H17" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="32" t="n">
+      <c r="I17" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="32" t="n">
+      <c r="J17" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="K17" s="32" t="n">
+      <c r="K17" s="37" t="n">
         <v>0.022</v>
       </c>
-      <c r="L17" s="32" t="n"/>
-      <c r="M17" s="32" t="n"/>
-      <c r="N17" s="32" t="n">
+      <c r="L17" s="37" t="n"/>
+      <c r="M17" s="37" t="n"/>
+      <c r="N17" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O17" s="32" t="n">
+      <c r="O17" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="P17" s="32" t="n">
+      <c r="P17" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q17" s="32" t="n">
+      <c r="Q17" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R17" s="32" t="n">
+      <c r="R17" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S17" s="32" t="n"/>
+      <c r="S17" s="37" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Monetizacion ', sección Banamex. TPV = B2 (8M) x C4 (35%). Share DEB Banamex B10 (TD), CRE B11 (TC). Débito B38, Crédito B39. Sobretasas MSI K39:K43. Sin AMEX/Internacional. 24x no aparece.</t>
@@ -1638,57 +1653,57 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Florence</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="30" t="n">
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="35" t="n">
         <v>4000000</v>
       </c>
-      <c r="E18" s="31" t="n">
+      <c r="E18" s="36" t="n">
         <v>60000</v>
       </c>
-      <c r="F18" s="32" t="n">
+      <c r="F18" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G18" s="32" t="n">
+      <c r="G18" s="37" t="n">
         <v>0.49</v>
       </c>
-      <c r="H18" s="32" t="n">
+      <c r="H18" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I18" s="32" t="n"/>
-      <c r="J18" s="32" t="n">
+      <c r="I18" s="37" t="n"/>
+      <c r="J18" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="K18" s="32" t="n">
+      <c r="K18" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="L18" s="32" t="n">
+      <c r="L18" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M18" s="32" t="n"/>
-      <c r="N18" s="32" t="n">
+      <c r="M18" s="37" t="n"/>
+      <c r="N18" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O18" s="32" t="n">
+      <c r="O18" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P18" s="32" t="n">
+      <c r="P18" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q18" s="32" t="n">
+      <c r="Q18" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R18" s="32" t="n"/>
-      <c r="S18" s="32" t="n"/>
+      <c r="R18" s="37" t="n"/>
+      <c r="S18" s="37" t="n"/>
       <c r="T18" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1696,57 +1711,57 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t>grupo_milano</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C19" s="29" t="n"/>
-      <c r="D19" s="30" t="n">
+      <c r="C19" s="34" t="n"/>
+      <c r="D19" s="35" t="n">
         <v>4000000</v>
       </c>
-      <c r="E19" s="31" t="n">
+      <c r="E19" s="36" t="n">
         <v>60000</v>
       </c>
-      <c r="F19" s="32" t="n">
+      <c r="F19" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G19" s="32" t="n">
+      <c r="G19" s="37" t="n">
         <v>0.49</v>
       </c>
-      <c r="H19" s="32" t="n">
+      <c r="H19" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I19" s="32" t="n"/>
-      <c r="J19" s="32" t="n">
+      <c r="I19" s="37" t="n"/>
+      <c r="J19" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="K19" s="32" t="n">
+      <c r="K19" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="L19" s="32" t="n">
+      <c r="L19" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M19" s="32" t="n"/>
-      <c r="N19" s="32" t="n">
+      <c r="M19" s="37" t="n"/>
+      <c r="N19" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O19" s="32" t="n">
+      <c r="O19" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P19" s="32" t="n">
+      <c r="P19" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q19" s="32" t="n">
+      <c r="Q19" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R19" s="32" t="n"/>
-      <c r="S19" s="32" t="n"/>
+      <c r="R19" s="37" t="n"/>
+      <c r="S19" s="37" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1754,57 +1769,57 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>Carlos Toys</t>
         </is>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="30" t="n">
+      <c r="C20" s="34" t="n"/>
+      <c r="D20" s="35" t="n">
         <v>4000000</v>
       </c>
-      <c r="E20" s="31" t="n">
+      <c r="E20" s="36" t="n">
         <v>60000</v>
       </c>
-      <c r="F20" s="32" t="n">
+      <c r="F20" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G20" s="32" t="n">
+      <c r="G20" s="37" t="n">
         <v>0.49</v>
       </c>
-      <c r="H20" s="32" t="n">
+      <c r="H20" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I20" s="32" t="n"/>
-      <c r="J20" s="32" t="n">
+      <c r="I20" s="37" t="n"/>
+      <c r="J20" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="K20" s="32" t="n">
+      <c r="K20" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="L20" s="32" t="n">
+      <c r="L20" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M20" s="32" t="n"/>
-      <c r="N20" s="32" t="n">
+      <c r="M20" s="37" t="n"/>
+      <c r="N20" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O20" s="32" t="n">
+      <c r="O20" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P20" s="32" t="n">
+      <c r="P20" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q20" s="32" t="n">
+      <c r="Q20" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R20" s="32" t="n"/>
-      <c r="S20" s="32" t="n"/>
+      <c r="R20" s="37" t="n"/>
+      <c r="S20" s="37" t="n"/>
       <c r="T20" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1812,57 +1827,57 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>Kaloni</t>
         </is>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C21" s="29" t="n"/>
-      <c r="D21" s="30" t="n">
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="35" t="n">
         <v>4000000</v>
       </c>
-      <c r="E21" s="31" t="n">
+      <c r="E21" s="36" t="n">
         <v>60000</v>
       </c>
-      <c r="F21" s="32" t="n">
+      <c r="F21" s="37" t="n">
         <v>0.43</v>
       </c>
-      <c r="G21" s="32" t="n">
+      <c r="G21" s="37" t="n">
         <v>0.49</v>
       </c>
-      <c r="H21" s="32" t="n">
+      <c r="H21" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="I21" s="32" t="n"/>
-      <c r="J21" s="32" t="n">
+      <c r="I21" s="37" t="n"/>
+      <c r="J21" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="K21" s="32" t="n">
+      <c r="K21" s="37" t="n">
         <v>0.018</v>
       </c>
-      <c r="L21" s="32" t="n">
+      <c r="L21" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M21" s="32" t="n"/>
-      <c r="N21" s="32" t="n">
+      <c r="M21" s="37" t="n"/>
+      <c r="N21" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O21" s="32" t="n">
+      <c r="O21" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P21" s="32" t="n">
+      <c r="P21" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q21" s="32" t="n">
+      <c r="Q21" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R21" s="32" t="n"/>
-      <c r="S21" s="32" t="n"/>
+      <c r="R21" s="37" t="n"/>
+      <c r="S21" s="37" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
           <t>Origen: Hoja1. Competidor no nombrado en el archivo ('Solución actual'). TPV = B2, ticket = B3, shares B5:B7 (MSI 10% B8 sin columna). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. ATENCIÓN: valores idénticos a Florence, grupo_milano, Carlos_Toys y Kaloni (posible plantilla copiada). Ticket 60,000 sospechoso.</t>
@@ -1870,63 +1885,63 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Bobois</t>
         </is>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C22" s="29" t="n"/>
-      <c r="D22" s="30" t="n">
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="35" t="n">
         <v>6000000</v>
       </c>
-      <c r="E22" s="31" t="n">
+      <c r="E22" s="36" t="n">
         <v>800</v>
       </c>
-      <c r="F22" s="32" t="n">
+      <c r="F22" s="37" t="n">
         <v>0.5</v>
       </c>
-      <c r="G22" s="32" t="n">
+      <c r="G22" s="37" t="n">
         <v>0.48</v>
       </c>
-      <c r="H22" s="32" t="n">
+      <c r="H22" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="I22" s="32" t="n">
+      <c r="I22" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="J22" s="32" t="n">
+      <c r="J22" s="37" t="n">
         <v>0.015</v>
       </c>
-      <c r="K22" s="32" t="n">
+      <c r="K22" s="37" t="n">
         <v>0.0185</v>
       </c>
-      <c r="L22" s="32" t="n">
+      <c r="L22" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="M22" s="32" t="n">
+      <c r="M22" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="N22" s="32" t="n">
+      <c r="N22" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="O22" s="32" t="n">
+      <c r="O22" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="P22" s="32" t="n">
+      <c r="P22" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q22" s="32" t="n">
+      <c r="Q22" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="R22" s="32" t="n">
+      <c r="R22" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S22" s="32" t="n"/>
+      <c r="S22" s="37" t="n"/>
       <c r="T22" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Escenario 24 horas '. Competidor no nombrado ('Solución actual'). TPV = B2 (6M), ticket = B3. Shares TD B5, TC B6, AMEX B7, Internacional = Débito B8 + Crédito B9 (0.5% + 0.5%). MSI 0% (B10). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%) - ambos 3.0%. Sobretasas MSI K17:K22 (3x con Citi 5% y 3x 5%; 18x 18.9%). 24x no aparece. Otras hojas (Escenario 1, 48 horas, citi 3x, Hoja2) tienen valores distintos.</t>
@@ -1934,57 +1949,57 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t>ARIAT</t>
         </is>
       </c>
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="30" t="n">
+      <c r="C23" s="34" t="n"/>
+      <c r="D23" s="35" t="n">
         <v>1800000</v>
       </c>
-      <c r="E23" s="31" t="n">
+      <c r="E23" s="36" t="n">
         <v>3800</v>
       </c>
-      <c r="F23" s="32" t="n">
+      <c r="F23" s="37" t="n">
         <v>0.19</v>
       </c>
-      <c r="G23" s="32" t="n">
+      <c r="G23" s="37" t="n">
         <v>0.8</v>
       </c>
-      <c r="H23" s="32" t="n">
+      <c r="H23" s="37" t="n">
         <v>0.01</v>
       </c>
-      <c r="I23" s="32" t="n"/>
-      <c r="J23" s="32" t="n">
+      <c r="I23" s="37" t="n"/>
+      <c r="J23" s="37" t="n">
         <v>0.025</v>
       </c>
-      <c r="K23" s="32" t="n">
+      <c r="K23" s="37" t="n">
         <v>0.025</v>
       </c>
-      <c r="L23" s="32" t="n">
+      <c r="L23" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M23" s="32" t="n"/>
-      <c r="N23" s="32" t="n">
+      <c r="M23" s="37" t="n"/>
+      <c r="N23" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O23" s="32" t="n">
+      <c r="O23" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P23" s="32" t="n">
+      <c r="P23" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q23" s="32" t="n">
+      <c r="Q23" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R23" s="32" t="n"/>
-      <c r="S23" s="32" t="n"/>
+      <c r="R23" s="37" t="n"/>
+      <c r="S23" s="37" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja '24h'. Competidor no nombrado ('Solución actual'). TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 1% B8 sin columna). Débito B17, Crédito B18, AMEX B19. Sobretasas MSI K17:K21. Sin Internacional, 18x ni 24x. Suma de shares = 101%. OP (TPV 400k) no incluido.</t>
@@ -1992,63 +2007,63 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>Petrolab</t>
         </is>
       </c>
-      <c r="B24" s="28" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C24" s="29" t="n"/>
-      <c r="D24" s="30" t="n">
+      <c r="C24" s="34" t="n"/>
+      <c r="D24" s="35" t="n">
         <v>4000000</v>
       </c>
-      <c r="E24" s="31" t="n">
+      <c r="E24" s="36" t="n">
         <v>1500</v>
       </c>
-      <c r="F24" s="32" t="n">
+      <c r="F24" s="37" t="n">
         <v>0.6</v>
       </c>
-      <c r="G24" s="32" t="n">
+      <c r="G24" s="37" t="n">
         <v>0.27</v>
       </c>
-      <c r="H24" s="32" t="n">
+      <c r="H24" s="37" t="n">
         <v>0.13</v>
       </c>
-      <c r="I24" s="32" t="n">
+      <c r="I24" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="32" t="n">
+      <c r="J24" s="37" t="n">
         <v>0.0191</v>
       </c>
-      <c r="K24" s="32" t="n">
+      <c r="K24" s="37" t="n">
         <v>0.0218</v>
       </c>
-      <c r="L24" s="32" t="n">
+      <c r="L24" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M24" s="32" t="n">
+      <c r="M24" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="N24" s="32" t="n">
+      <c r="N24" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="O24" s="32" t="n">
+      <c r="O24" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="P24" s="32" t="n">
+      <c r="P24" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q24" s="32" t="n">
+      <c r="Q24" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="R24" s="32" t="n">
+      <c r="R24" s="37" t="n">
         <v>0.189</v>
       </c>
-      <c r="S24" s="32" t="n"/>
+      <c r="S24" s="37" t="n"/>
       <c r="T24" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Hoja1'. Competidor no nombrado ('Solución actual'). TPV = B2 ('Procesamiento'), ticket = B3. Shares TD B5, TC B6, AMEX B7, Int = Débito B8 + Crédito B9 (0%). Débito B17, Crédito B18, AMEX B19, Int Crédito B20 (3.0%), Int Débito B21 (3.0%). Sobretasas MSI J17:J22. 24x no aparece. OP (TPV 100k) no incluido.</t>
@@ -2056,63 +2071,63 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t>Reina Diaz</t>
         </is>
       </c>
-      <c r="B25" s="28" t="inlineStr">
+      <c r="B25" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C25" s="29" t="n"/>
-      <c r="D25" s="30" t="n">
+      <c r="C25" s="34" t="n"/>
+      <c r="D25" s="35" t="n">
         <v>800000</v>
       </c>
-      <c r="E25" s="31" t="n">
+      <c r="E25" s="36" t="n">
         <v>3800</v>
       </c>
-      <c r="F25" s="32" t="n">
+      <c r="F25" s="37" t="n">
         <v>0.2</v>
       </c>
-      <c r="G25" s="32" t="n">
+      <c r="G25" s="37" t="n">
         <v>0.79</v>
       </c>
-      <c r="H25" s="32" t="n">
+      <c r="H25" s="37" t="n">
         <v>0.02</v>
       </c>
-      <c r="I25" s="32" t="n">
+      <c r="I25" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="32" t="n">
+      <c r="J25" s="37" t="n">
         <v>0.0169</v>
       </c>
-      <c r="K25" s="32" t="n">
+      <c r="K25" s="37" t="n">
         <v>0.0213</v>
       </c>
-      <c r="L25" s="32" t="n">
+      <c r="L25" s="37" t="n">
         <v>0.0285</v>
       </c>
-      <c r="M25" s="32" t="n">
+      <c r="M25" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="N25" s="32" t="n">
+      <c r="N25" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="O25" s="32" t="n">
+      <c r="O25" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="P25" s="32" t="n">
+      <c r="P25" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q25" s="32" t="n">
+      <c r="Q25" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="R25" s="32" t="n">
+      <c r="R25" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S25" s="32" t="n">
+      <c r="S25" s="37" t="n">
         <v>0.189</v>
       </c>
       <c r="T25" s="7" t="inlineStr">
@@ -2122,59 +2137,59 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>JULIO CEPEDA</t>
         </is>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C26" s="29" t="n"/>
-      <c r="D26" s="30" t="n">
+      <c r="C26" s="34" t="n"/>
+      <c r="D26" s="35" t="n">
         <v>1000000</v>
       </c>
-      <c r="E26" s="31" t="n">
+      <c r="E26" s="36" t="n">
         <v>700</v>
       </c>
-      <c r="F26" s="32" t="n">
+      <c r="F26" s="37" t="n">
         <v>0.33</v>
       </c>
-      <c r="G26" s="32" t="n">
+      <c r="G26" s="37" t="n">
         <v>0.4</v>
       </c>
-      <c r="H26" s="32" t="n">
+      <c r="H26" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="I26" s="32" t="n"/>
-      <c r="J26" s="32" t="n">
+      <c r="I26" s="37" t="n"/>
+      <c r="J26" s="37" t="n">
         <v>0.0137</v>
       </c>
-      <c r="K26" s="32" t="n">
+      <c r="K26" s="37" t="n">
         <v>0.019</v>
       </c>
-      <c r="L26" s="32" t="n">
+      <c r="L26" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M26" s="32" t="n"/>
-      <c r="N26" s="32" t="n">
+      <c r="M26" s="37" t="n"/>
+      <c r="N26" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O26" s="32" t="n">
+      <c r="O26" s="37" t="n">
         <v>0.0395</v>
       </c>
-      <c r="P26" s="32" t="n">
+      <c r="P26" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q26" s="32" t="n">
+      <c r="Q26" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="R26" s="32" t="n">
+      <c r="R26" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="S26" s="32" t="n"/>
+      <c r="S26" s="37" t="n"/>
       <c r="T26" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Sin MSIs'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B6, TC B7, AMEX B8 (MSI 3% B9 sin columna). Débito B13, Crédito B14, AMEX B15. Sobretasas MSI K13:K17 (3x con Citi 3.2%, 3x 3.95%). Sin Internacional, 18x ni 24x. Suma de shares = 86%. Hoja 'MSIs' no revisada.</t>
@@ -2182,63 +2197,63 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>2CAP (Nacional)</t>
         </is>
       </c>
-      <c r="B27" s="28" t="inlineStr">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C27" s="29" t="n"/>
-      <c r="D27" s="30" t="n">
+      <c r="C27" s="34" t="n"/>
+      <c r="D27" s="35" t="n">
         <v>15000000</v>
       </c>
-      <c r="E27" s="31" t="n">
+      <c r="E27" s="36" t="n">
         <v>1100</v>
       </c>
-      <c r="F27" s="32" t="n">
+      <c r="F27" s="37" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="G27" s="32" t="n">
+      <c r="G27" s="37" t="n">
         <v>0.38</v>
       </c>
-      <c r="H27" s="32" t="n">
+      <c r="H27" s="37" t="n">
         <v>0.02</v>
       </c>
-      <c r="I27" s="32" t="n">
+      <c r="I27" s="37" t="n">
         <v>0.04</v>
       </c>
-      <c r="J27" s="32" t="n">
+      <c r="J27" s="37" t="n">
         <v>0.014</v>
       </c>
-      <c r="K27" s="32" t="n">
+      <c r="K27" s="37" t="n">
         <v>0.015</v>
       </c>
-      <c r="L27" s="32" t="n">
+      <c r="L27" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="M27" s="32" t="n">
+      <c r="M27" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="N27" s="32" t="n">
+      <c r="N27" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O27" s="32" t="n">
+      <c r="O27" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P27" s="32" t="n">
+      <c r="P27" s="37" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="Q27" s="32" t="n">
+      <c r="Q27" s="37" t="n">
         <v>0.115</v>
       </c>
-      <c r="R27" s="32" t="n">
+      <c r="R27" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S27" s="32" t="n"/>
+      <c r="S27" s="37" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Monetizacion Aeropuerto T7', bloque 'Procesamiento Actual en terminales' (B2:B11). Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int Débito B8 (MSI 5% B11 sin columna). Débito B24, Crédito B25, AMEX B26, Int B27. Sobretasas MSI J24:J29. 24x no aparece. Otras hojas (T4, T2, 2/4/7 DIAS) no revisadas.</t>
@@ -2246,63 +2261,63 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t>2CAP (Aeropuerto T7)</t>
         </is>
       </c>
-      <c r="B28" s="28" t="inlineStr">
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="30" t="n">
+      <c r="C28" s="34" t="n"/>
+      <c r="D28" s="35" t="n">
         <v>8000000</v>
       </c>
-      <c r="E28" s="31" t="n">
+      <c r="E28" s="36" t="n">
         <v>1800</v>
       </c>
-      <c r="F28" s="32" t="n">
+      <c r="F28" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="G28" s="32" t="n">
+      <c r="G28" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="H28" s="32" t="n">
+      <c r="H28" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="I28" s="32" t="n">
+      <c r="I28" s="37" t="n">
         <v>0.7</v>
       </c>
-      <c r="J28" s="32" t="n">
+      <c r="J28" s="37" t="n">
         <v>0.014</v>
       </c>
-      <c r="K28" s="32" t="n">
+      <c r="K28" s="37" t="n">
         <v>0.015</v>
       </c>
-      <c r="L28" s="32" t="n">
+      <c r="L28" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="M28" s="32" t="n">
+      <c r="M28" s="37" t="n">
         <v>0.029</v>
       </c>
-      <c r="N28" s="32" t="n">
+      <c r="N28" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O28" s="32" t="n">
+      <c r="O28" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P28" s="32" t="n">
+      <c r="P28" s="37" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="Q28" s="32" t="n">
+      <c r="Q28" s="37" t="n">
         <v>0.115</v>
       </c>
-      <c r="R28" s="32" t="n">
+      <c r="R28" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S28" s="32" t="n"/>
+      <c r="S28" s="37" t="n"/>
       <c r="T28" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Monetizacion Aeropuerto T7', bloque 'Procesamiento Actual en Aeropuertos' (D2:E9). TPV = E2, ticket = E3. Shares TD E5, TC E6, AMEX E7, Int Débito E8 = 70% (revisar, parece alto). Tasas B36:B39 y sobretasas J36:J41 iguales al nacional. 24x no aparece.</t>
@@ -2310,57 +2325,57 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>Dega</t>
         </is>
       </c>
-      <c r="B29" s="28" t="inlineStr">
+      <c r="B29" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C29" s="29" t="n"/>
-      <c r="D29" s="30" t="n">
+      <c r="C29" s="34" t="n"/>
+      <c r="D29" s="35" t="n">
         <v>2500000</v>
       </c>
-      <c r="E29" s="31" t="n">
+      <c r="E29" s="36" t="n">
         <v>4500</v>
       </c>
-      <c r="F29" s="32" t="n">
+      <c r="F29" s="37" t="n">
         <v>0.34</v>
       </c>
-      <c r="G29" s="32" t="n">
+      <c r="G29" s="37" t="n">
         <v>0.61</v>
       </c>
-      <c r="H29" s="32" t="n">
+      <c r="H29" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="I29" s="32" t="n"/>
-      <c r="J29" s="32" t="n">
+      <c r="I29" s="37" t="n"/>
+      <c r="J29" s="37" t="n">
         <v>0.0117</v>
       </c>
-      <c r="K29" s="32" t="n">
+      <c r="K29" s="37" t="n">
         <v>0.0155</v>
       </c>
-      <c r="L29" s="32" t="n">
+      <c r="L29" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M29" s="32" t="n"/>
-      <c r="N29" s="32" t="n">
+      <c r="M29" s="37" t="n"/>
+      <c r="N29" s="37" t="n">
         <v>0.032</v>
       </c>
-      <c r="O29" s="32" t="n">
+      <c r="O29" s="37" t="n">
         <v>0.055</v>
       </c>
-      <c r="P29" s="32" t="n">
+      <c r="P29" s="37" t="n">
         <v>0.08699999999999999</v>
       </c>
-      <c r="Q29" s="32" t="n">
+      <c r="Q29" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="R29" s="32" t="n"/>
-      <c r="S29" s="32" t="n"/>
+      <c r="R29" s="37" t="n"/>
+      <c r="S29" s="37" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Hoja1'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7 (MSI 8% B8 sin columna; la suma TD+TC+AMEX+MSI = 108%, revisar). Débito B12, Crédito B13, AMEX B14. Sobretasas MSI J12:J16. Sin Internacional, 18x ni 24x. OP no incluido.</t>
@@ -2368,63 +2383,63 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>dENTISTA</t>
         </is>
       </c>
-      <c r="B30" s="28" t="inlineStr">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>No identificado</t>
         </is>
       </c>
-      <c r="C30" s="29" t="n"/>
-      <c r="D30" s="30" t="n">
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="35" t="n">
         <v>2500000</v>
       </c>
-      <c r="E30" s="31" t="n">
+      <c r="E30" s="36" t="n">
         <v>3000</v>
       </c>
-      <c r="F30" s="32" t="n">
+      <c r="F30" s="37" t="n">
         <v>0.3795</v>
       </c>
-      <c r="G30" s="32" t="n">
+      <c r="G30" s="37" t="n">
         <v>0.2192</v>
       </c>
-      <c r="H30" s="32" t="n">
+      <c r="H30" s="37" t="n">
         <v>0.0213</v>
       </c>
-      <c r="I30" s="32" t="n">
+      <c r="I30" s="37" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="J30" s="32" t="n">
+      <c r="J30" s="37" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="K30" s="32" t="n">
+      <c r="K30" s="37" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="L30" s="32" t="n">
+      <c r="L30" s="37" t="n">
         <v>0.0293</v>
       </c>
-      <c r="M30" s="32" t="n">
+      <c r="M30" s="37" t="n">
         <v>0.014</v>
       </c>
-      <c r="N30" s="32" t="n">
+      <c r="N30" s="37" t="n">
         <v>0.0485</v>
       </c>
-      <c r="O30" s="32" t="n">
+      <c r="O30" s="37" t="n">
         <v>0.074</v>
       </c>
-      <c r="P30" s="32" t="n">
+      <c r="P30" s="37" t="n">
         <v>0.099</v>
       </c>
-      <c r="Q30" s="32" t="n">
+      <c r="Q30" s="37" t="n">
         <v>0.129</v>
       </c>
-      <c r="R30" s="32" t="n">
+      <c r="R30" s="37" t="n">
         <v>0.189</v>
       </c>
-      <c r="S30" s="32" t="n"/>
+      <c r="S30" s="37" t="n"/>
       <c r="T30" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja 'Hoja1'. Competidor no nombrado. TPV = B2, ticket = B3. Shares TD B5, TC B6, AMEX B7, Int = Débito B8 + Crédito B9 (3.5% + 3.5%). MSI 31% (B10) sin columna. Débito B15, Crédito B16, AMEX B17, Int Crédito B18 (1.4%), Int Débito B19 (1.4%). Sobretasas MSI J15:J20 (3x con Citi = 3x = 4.85%). Sin 24x. Tasa TD/TC (0.9%) muy baja, revisar.</t>
@@ -2432,63 +2447,63 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="33" t="inlineStr">
         <is>
           <t>APEC</t>
         </is>
       </c>
-      <c r="B31" s="28" t="inlineStr">
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>BBVA</t>
         </is>
       </c>
-      <c r="C31" s="29" t="n"/>
-      <c r="D31" s="30" t="n">
+      <c r="C31" s="34" t="n"/>
+      <c r="D31" s="35" t="n">
         <v>21780000</v>
       </c>
-      <c r="E31" s="31" t="n">
+      <c r="E31" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F31" s="32" t="n">
+      <c r="F31" s="37" t="n">
         <v>0.373</v>
       </c>
-      <c r="G31" s="32" t="n">
+      <c r="G31" s="37" t="n">
         <v>0.16</v>
       </c>
-      <c r="H31" s="32" t="n">
+      <c r="H31" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="32" t="n">
+      <c r="I31" s="37" t="n">
         <v>0.007</v>
       </c>
-      <c r="J31" s="32" t="n">
+      <c r="J31" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="K31" s="32" t="n">
+      <c r="K31" s="37" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="L31" s="32" t="n">
+      <c r="L31" s="37" t="n">
         <v>0.03</v>
       </c>
-      <c r="M31" s="32" t="n">
+      <c r="M31" s="37" t="n">
         <v>0.0225</v>
       </c>
-      <c r="N31" s="32" t="n">
+      <c r="N31" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O31" s="32" t="n">
+      <c r="O31" s="37" t="n">
         <v>0.075</v>
       </c>
-      <c r="P31" s="32" t="n">
+      <c r="P31" s="37" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q31" s="32" t="n">
+      <c r="Q31" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="R31" s="32" t="n">
+      <c r="R31" s="37" t="n">
         <v>0.18</v>
       </c>
-      <c r="S31" s="32" t="n"/>
+      <c r="S31" s="37" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Monetizacion 0.60%'. TPV = B3 (B2 x C3 = 66%). Shares TD B7, TC B8, Int B14 (7%, total). BBVA MSI 10% (B9) sin columna. Débito B25 = 0% (revisar; la tasa base TC aparece como 0.99% en J25:J30), Crédito B26, AMEX B27, Int B28. Sobretasas MSI K25:K30. 24x no aparece. TPV sin periodo (tratado como mensual).</t>
@@ -2496,55 +2511,55 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>APEC</t>
         </is>
       </c>
-      <c r="B32" s="28" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>Scotia</t>
         </is>
       </c>
-      <c r="C32" s="29" t="n"/>
-      <c r="D32" s="30" t="n">
+      <c r="C32" s="34" t="n"/>
+      <c r="D32" s="35" t="n">
         <v>11220000</v>
       </c>
-      <c r="E32" s="31" t="n">
+      <c r="E32" s="36" t="n">
         <v>555</v>
       </c>
-      <c r="F32" s="32" t="n">
+      <c r="F32" s="37" t="n">
         <v>0.06</v>
       </c>
-      <c r="G32" s="32" t="n">
+      <c r="G32" s="37" t="n">
         <v>0.06</v>
       </c>
-      <c r="H32" s="32" t="n"/>
-      <c r="I32" s="32" t="n"/>
-      <c r="J32" s="32" t="n">
+      <c r="H32" s="37" t="n"/>
+      <c r="I32" s="37" t="n"/>
+      <c r="J32" s="37" t="n">
         <v>0.012</v>
       </c>
-      <c r="K32" s="32" t="n">
+      <c r="K32" s="37" t="n">
         <v>0.012</v>
       </c>
-      <c r="L32" s="32" t="n"/>
-      <c r="M32" s="32" t="n"/>
-      <c r="N32" s="32" t="n">
+      <c r="L32" s="37" t="n"/>
+      <c r="M32" s="37" t="n"/>
+      <c r="N32" s="37" t="n">
         <v>0.035</v>
       </c>
-      <c r="O32" s="32" t="n">
+      <c r="O32" s="37" t="n">
         <v>0.045</v>
       </c>
-      <c r="P32" s="32" t="n">
+      <c r="P32" s="37" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q32" s="32" t="n">
+      <c r="Q32" s="37" t="n">
         <v>0.095</v>
       </c>
-      <c r="R32" s="32" t="n">
+      <c r="R32" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="S32" s="32" t="n"/>
+      <c r="S32" s="37" t="n"/>
       <c r="T32" s="7" t="inlineStr">
         <is>
           <t>Origen: hoja activa 'Monetizacion 0.60%', sección Scotia (B4 'mifel' = 34%, TPV = B4). Shares DEB SCOTIA B10 (TD), CRE SCOTIA B11 (TC), MSI SCOTIA 22% (B13) sin columna. Débito B38, Crédito B39. Sobretasas MSI K39:K43. 6x = 4.5% (K40); 6x con Citibanamex = 8.76% (K38) no mapeada. Sin AMEX/Internacional. 24x no aparece.</t>
@@ -3019,6 +3034,96 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="38" t="inlineStr">
+        <is>
+          <t>Svenson</t>
+        </is>
+      </c>
+      <c r="B42" s="38" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t>Clínicas Salud (truncada en foto)</t>
+        </is>
+      </c>
+      <c r="D42" s="40" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="42" t="n"/>
+      <c r="G42" s="42" t="n"/>
+      <c r="H42" s="42" t="n"/>
+      <c r="I42" s="42" t="n"/>
+      <c r="J42" s="42" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="K42" s="42" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="L42" s="42" t="n"/>
+      <c r="M42" s="42" t="n"/>
+      <c r="N42" s="42" t="n">
+        <v>0.0492</v>
+      </c>
+      <c r="O42" s="42" t="n">
+        <v>0.08409999999999999</v>
+      </c>
+      <c r="P42" s="42" t="n"/>
+      <c r="Q42" s="42" t="n">
+        <v>0.1489</v>
+      </c>
+      <c r="R42" s="42" t="n"/>
+      <c r="S42" s="42" t="n"/>
+      <c r="T42" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto (hoja compartida). Débito 1.75%, Crédito 2.38%, AMEX vacío. MSI: 3x 4.92%, 6x 8.41%, 9x NA, 12x 14.89%, 18x NA. Costo fijo: No. Liberación: día siguiente. Ligas de pago: No. Sin TPV ni shares en la foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="inlineStr">
+        <is>
+          <t>Muebleria Corra</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D43" s="40" t="n"/>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="42" t="n"/>
+      <c r="G43" s="42" t="n"/>
+      <c r="H43" s="42" t="n"/>
+      <c r="I43" s="42" t="n"/>
+      <c r="J43" s="42" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K43" s="42" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="L43" s="42" t="n"/>
+      <c r="M43" s="42" t="n"/>
+      <c r="N43" s="42" t="n"/>
+      <c r="O43" s="42" t="n"/>
+      <c r="P43" s="42" t="n"/>
+      <c r="Q43" s="42" t="n"/>
+      <c r="R43" s="42" t="n"/>
+      <c r="S43" s="42" t="n"/>
+      <c r="T43" s="7" t="inlineStr">
+        <is>
+          <t>Dato de foto. Débito se ve como '0,01' sin % (guardé 1%, confirmar). Crédito 1.35%, AMEX NA. MSI: 'Hasta 12 MS arr...' cortado en la foto, sin tasas por plazo. Costo fijo: No.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>